<commit_message>
Round 6 (Codex + Cursor final review): soften unphased diagnosis wording, fix 313-residue phrasing, 2.59x score ratio, remove duplicated Q23 block, tone in Track 2 abstract
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MzYcL5yWqm6WtVGNokxBZa
</commit_message>
<xml_diff>
--- a/submission/methods_description_form_ciberpty.xlsx
+++ b/submission/methods_description_form_ciberpty.xlsx
@@ -527,6 +527,7 @@
     </row>
     <row r="3"/>
     <row r="4"/>
+    <row r="5"/>
     <row r="6" ht="16" customHeight="1" s="7">
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -567,7 +568,7 @@
       <c r="B9" s="3" t="inlineStr">
         <is>
           <t>We ran two independent analyses and required them to converge before accepting a result.
-### Analysis A — phenotype-driven, genome-wide, hypothesis-free (primary)
+### Analysis A — genome-wide, phenotype-informed, hypothesis-free (primary)
 Exomiser 15.1.0 with the 2602 hg38 and 2602 phenotype data releases. Input was the unmodified proband
 VCF — 5,012,204 records, of which 4,740,790 carry the PASS filter (GRCh38, GATK 4.2.4.0) — together
 with the eight HPO terms extracted verbatim from the supplied clinical document:
@@ -605,7 +606,7 @@
 dominant colorectal cancer diagnosis. The result we stand behind is rank 2, not rank 1. We say so
 because the honest reading of our own output matters more than the better-sounding headline.
 The combined score gap is real but moderate: 0.5871 (rank 1, AD) and 0.5538 (rank 2, AR) against
-0.2137 for the third-ranked gene — 2.75× the third gene, not an order of magnitude.
+0.2137 for the third-ranked gene — 2.59× the third gene for the recessive result we stand behind (2.75× for the dominant artefact), not an order of magnitude.
 ### Robustness controls — including one that argues against us
 We ran eleven additional Exomiser analyses to test how much of the result comes from the phenotype
 and how much from the variant.
@@ -732,14 +733,7 @@
 No block of the VCF and no genotype table was ever sent to a language model. All genomic work ran
 on local tools (bcftools, Exomiser 15.1.0) and on annotation APIs — Ensembl VEP and ClinVar — that
 the hackathon policy names explicitly as acceptable. What the models saw were named variants, HPO
-terms and reasoning: exactly the category the policy classifies as a "finding" and permits retaining.
----
-The factual statement above holds regardless of tooling details:
-No block of the VCF and no genotype table was ever sent to a large language model. All genomic
-work ran on local tools (bcftools, Exomiser 15.1.0) and on annotation APIs — Ensembl VEP and
-ClinVar — that the hackathon policy names explicitly as acceptable. What the language models saw were
-named variants, HPO terms and reasoning: exactly the category the policy classifies as a "finding"
-and permits retaining.</t>
+terms and reasoning: exactly the category the policy classifies as a "finding" and permits retaining.</t>
         </is>
       </c>
     </row>
@@ -956,8 +950,7 @@
 Limitations. Phase cannot be established: no parental sample, and the variants lie ~11 kb apart,
 beyond read-backed phasing (confirmed by the absence of GATK phase tags on both). The functional
 consequence of p.Asn1002Lys is unproven, and its in-silico predictors disagree (REVEL 0.472,
-AlphaMissense 0.923). REMM and CADD were omitted. Total analysis time was 53 seconds on a commodity
-workstation with no GPU.</t>
+AlphaMissense 0.923). REMM and CADD were omitted. The genome-wide Exomiser run took 53 seconds on a commodity workstation with no GPU.</t>
         </is>
       </c>
     </row>
@@ -1000,6 +993,7 @@
     </row>
     <row r="3"/>
     <row r="4"/>
+    <row r="5"/>
     <row r="6" ht="16" customHeight="1" s="7">
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -1029,10 +1023,8 @@
         <is>
           <t>We went from variant to candidate in five steps, and the third and fifth are where most candidates die.
 Step 1 — establish the lesion. Compound heterozygosity in BUB1B: c.2210T&gt;G p.Leu737Ter, a
-nonsense allele truncating 313 residues before the C-terminal kinase domain (UniProt O60566 annotates
-it at 766–1050), paired with c.3006T&gt;G p.Asn1002Lys inside that domain. Loss of function, matching
-the truncating-plus-missense pattern of viable MVA1: a null allele with a hypomorphic one, biallelic
-null being lethal.
+nonsense allele that removes the C-terminal 313 residues, including the kinase domain (UniProt O60566 annotates it at 766–1050), paired with c.3006T&gt;G p.Asn1002Lys inside that domain. Loss of function, matching
+the truncating-plus-missense pattern of viable MVA1: a null allele with a hypomorphic one. Reading the pair as null-plus-hypomorph is our inference from PMID 20516114; that source does not state that complete biallelic loss is lethal, and neither do we.
 Step 2 — follow the mechanism downstream, not at the lesion. No approved drug restores BubR1.
 We therefore asked what the lesion produces that is druggable. The chain is: weakened spindle
 assembly checkpoint → chromosome mis-segregation → constitutional aneuploidy → stoichiometric
@@ -1180,7 +1172,7 @@
         <is>
           <t>Loss of function, with the druggable target displaced downstream of the lesion.
 The nonsense allele removes the entire C-terminal kinase domain; the missense allele sits inside it.
-cell lines derived from MVA patients with biallelic mutations show "an impaired mitotic checkpoint,
+Cell lines derived from MVA patients with biallelic mutations show "an impaired mitotic checkpoint,
 chromosome alignment defects, and low overall BUBR1 abundance" (PMID 20516114), and allele-specific effects — not merely total BubR1 quantity — drive phenotypic
 heterogeneity (Sieben 2020, PMID 31738183).
 We were explicit about what we could not determine. Phase is not established: no parental
@@ -1256,8 +1248,8 @@
 Limitations. The proteasome dependency is established in cancer aneuploidy, not constitutional
 mosaicism; whether it transfers is precisely what our eight-week experiment tests, and we
 have not assumed it. The EC50 is a conservative bound read from a figure panel. Phase is unproven.
-And the honest answer to "what should he take today" is nothing — the intervention that most changes
-his prognosis now is surveillance, not a molecule.</t>
+And no disease-modifying drug can be recommended from these data today — the intervention that most
+changes his prognosis now is surveillance, not a molecule.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Track 2 round 7: AACR 2024 MVA surveillance consensus, 2026 CRISPR/case-report evidence, family one-pager, five-filter funnel figure and reusable worksheet
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MzYcL5yWqm6WtVGNokxBZa
</commit_message>
<xml_diff>
--- a/submission/methods_description_form_ciberpty.xlsx
+++ b/submission/methods_description_form_ciberpty.xlsx
@@ -1101,10 +1101,12 @@
         <is>
           <t>Three activities, all documented in the repository:
 1. Citation verification. Every PMID was checked against PubMed or Europe PMC before use. This
-   was not ceremonial: three fabricated or misattributed citations were caught and removed —
-   a paper on acromegaly cited as Wilms surveillance (PMID 17652220, replaced by 16857697), a TRIP13
-   paper cited for the BUB1B tumour spectrum (PMID 28553959), and two KARD papers merged under one
-   attribution (separated into PMID 23789096 and 23345399).
+   was not ceremonial: three citation problems were caught, of three different kinds —
+   one wrong paper (a study of acromegaly cited as Wilms surveillance, PMID 17652220, replaced by
+   16857697); one merged attribution (two KARD papers under a single citation, separated into
+   PMID 23789096 and 23345399); and one over-extension (PMID 28553959 was being used to carry the
+   proteotoxic rationale to CEP57, which that same source contradicts — we withdrew that use and kept
+   the paper only for the BUB1B/TRIP13 embryonal-tumour sentence its abstract actually states).
 2. Adversarial review by independent models. Two different language models were asked to attack
    our own drafts. They found, among others, a claim of ours that contradicted our own data file:
    the report stated that Tang et al. used only stable trisomies, when our extraction record shows

</xml_diff>

<commit_message>
Round 7 corrections: fix contaminated unrelated-HPO control (two terms were annotated to MVA1), re-run with verified terms (BUB1B still rank 1, score 0.4187); resolve four contradictions introduced by the Track 2 revision
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MzYcL5yWqm6WtVGNokxBZa
</commit_message>
<xml_diff>
--- a/submission/methods_description_form_ciberpty.xlsx
+++ b/submission/methods_description_form_ciberpty.xlsx
@@ -608,16 +608,30 @@
 The combined score gap is real but moderate: 0.5871 (rank 1, AD) and 0.5538 (rank 2, AR) against
 0.2137 for the third-ranked gene — 2.59× the third gene for the recessive result we stand behind (2.75× for the dominant artefact), not an order of magnitude.
 ### Robustness controls — including one that argues against us
-We ran eleven additional Exomiser analyses to test how much of the result comes from the phenotype
+We ran twelve additional Exomiser analyses to test how much of the result comes from the phenotype
 and how much from the variant.
 Leave-one-HPO-out (8 runs). Removing each HPO term in turn: BUB1B remained rank 1 in all
 eight, with scores from 0.5447 to 0.7503. Removing the rhabdomyosarcoma term — the one a human
 would consider most diagnostic — actually raised the score to 0.7503. No single symptom carries the
 result.
-Unrelated HPO terms (1 run). Replacing the eight clinical terms with five clinically unrelated
-ones — seizure (HP:0001250), hearing impairment (HP:0000365), atrial septal defect (HP:0001631),
-conjunctivitis (HP:0000509) and recurrent respiratory infections (HP:0002205) — BUB1B still came
-out rank 1, score 0.5506.
+Unrelated HPO terms (2 runs, one of which corrects the other). Our first version of this control
+replaced the eight clinical terms with five we described as "clinically unrelated" — seizure
+(HP:0001250), hearing impairment (HP:0000365), atrial septal defect (HP:0001631), conjunctivitis
+(HP:0000509) and recurrent respiratory infections (HP:0002205). BUB1B came out rank 1, score 0.5506.
+That control was contaminated, and we caught it ourselves. Querying the HPO annotations for
+OMIM:257300 returns 59 terms, and two of our five are among them: seizure (HP:0001250, Nervous
+System) and atrial septal defect (HP:0001631, Cardiovascular). Congenital heart defects including
+septal defects are an established feature of MVA, and BubR1 loss disrupts cardiac development
+(PMID 40055864). So the run was not a phenotype-free control at all — it fed the pipeline two genuine
+MVA features.
+We re-ran it with five terms verified against the same annotation set as absent from MVA1: hearing
+impairment (HP:0000365), conjunctivitis (HP:0000509), recurrent respiratory infections (HP:0002205),
+headache (HP:0002315) and pruritus (HP:0000989). BUB1B still came out rank 1 of 4,565 genes, score
+0.4187. The conclusion survives a clean control.
+The comparison is itself informative. Removing the two contaminating terms drops the score from 0.5506
+to 0.4187 — about 24% — without changing the rank. That is the size of the phenotype's contribution
+here: measurable, and not enough to decide the answer. Script and log:
+`tools/control_hpo_r7.sh`, `tools/logs/controles_hpo_r7.log`.
 Least-specific term alone (1 run). With short stature (HP:0004322) as the only input, BUB1B fell
 to rank 4 and HK1 took the top slot.
 No phenotype at all (1 run). Exomiser terminates with an error; the tool requires at least one
@@ -897,7 +911,7 @@
       <c r="B18" s="3" t="inlineStr">
         <is>
           <t>- Exomiser genome-wide run: 53 seconds wall clock (32-core CPU, 16 GB JVM heap).
-- Eleven robustness controls: about 10 minutes total.
+- Twelve robustness controls: about 10 minutes total.
 - Targeted panel with REST annotation: under 5 minutes, dominated by API latency.
 - Mosaicism analysis: about 10 minutes of bcftools streaming.
 - One-off setup: ≈55 GB of Exomiser reference data downloaded and extracted.
@@ -935,7 +949,7 @@
 Pathogenic/Likely pathogenic; gnomAD 9.98×10⁻⁵) and c.3006T&gt;G p.Asn1002Lys (missense; gnomAD
 8.99×10⁻⁷; not in ClinVar), consistent with MVA1 (OMIM 257300) and with the truncating-plus-missense
 allelic pattern of viable MVA1.
-Eleven robustness controls, one of which argues against us. Leave-one-HPO-out keeps BUB1B at rank
+Twelve robustness controls, one of which argues against us. Leave-one-HPO-out keeps BUB1B at rank
 1 in all eight runs, so no single symptom drives the result — but substituting clinically unrelated
 HPO terms also returns BUB1B at rank 1. We therefore describe the finding as variant-driven and
 phenotype-consistent, not phenotype-driven: the ClinVar-whitelisted nonsense allele carries the
@@ -993,7 +1007,6 @@
     </row>
     <row r="3"/>
     <row r="4"/>
-    <row r="5"/>
     <row r="6" ht="16" customHeight="1" s="7">
       <c r="B6" s="1" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Round 7 consistency pass: align the family page, closing note and methods form with the revised metformin verdict and the honest scope of the fibroblast experiment
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MzYcL5yWqm6WtVGNokxBZa
</commit_message>
<xml_diff>
--- a/submission/methods_description_form_ciberpty.xlsx
+++ b/submission/methods_description_form_ciberpty.xlsx
@@ -1007,6 +1007,7 @@
     </row>
     <row r="3"/>
     <row r="4"/>
+    <row r="5"/>
     <row r="6" ht="16" customHeight="1" s="7">
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -1037,7 +1038,7 @@
           <t>We went from variant to candidate in five steps, and the third and fifth are where most candidates die.
 Step 1 — establish the lesion. Compound heterozygosity in BUB1B: c.2210T&gt;G p.Leu737Ter, a
 nonsense allele that removes the C-terminal 313 residues, including the kinase domain (UniProt O60566 annotates it at 766–1050), paired with c.3006T&gt;G p.Asn1002Lys inside that domain. Loss of function, matching
-the truncating-plus-missense pattern of viable MVA1: a null allele with a hypomorphic one. Reading the pair as null-plus-hypomorph is our inference from PMID 20516114; that source does not state that complete biallelic loss is lethal, and neither do we.
+the truncating-plus-missense pattern of viable MVA1: a null allele with a hypomorphic one. Reading the pair as null-plus-hypomorph is our reading of the human truncating-plus-missense pattern (PMID 20516114), which does not state that complete biallelic loss is lethal, and neither do we; the separate prediction that p.Asn1002Lys retains more residual function than L1012P comes from the Sieben mouse series (PMID 31738183), not from 20516114.
 Step 2 — follow the mechanism downstream, not at the lesion. No approved drug restores BubR1.
 We therefore asked what the lesion produces that is druggable. The chain is: weakened spindle
 assembly checkpoint → chromosome mis-segregation → constitutional aneuploidy → stoichiometric
@@ -1063,7 +1064,7 @@
 filter 4 for this child, which is a patient-specific verdict rather than a property of the drug.
 We state the condition under which it would become appropriate — an MVA patient with an active
 tumour, where the comparator is cytotoxic chemotherapy rather than nothing — and we propose an
-eight-week experiment that could falsify the whole proposal.</t>
+experiment — an eight-week assay window, about twelve weeks from a fresh biopsy — that could fail to support the dependency in this child's own cells. It would not, on its own, close the tumour-board question, and we say so where we describe it.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync the methods form and the Track 2 mirror to the round-8 corrections
Track 1 sheet: Q3 and the Q12 abstract regenerated from the corrected report (abstract
496/500). Track 2 sheet: the mechanism answer and the abstract now carry the measured
phasing result and the fact that the retrieval pipeline is insensitive to phase
(abstract trimmed back to 500/500). methods_track2.md regenerated from the sheet so the
two stay mirrors.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MzYcL5yWqm6WtVGNokxBZa
</commit_message>
<xml_diff>
--- a/submission/methods_description_form_ciberpty.xlsx
+++ b/submission/methods_description_form_ciberpty.xlsx
@@ -527,7 +527,6 @@
     </row>
     <row r="3"/>
     <row r="4"/>
-    <row r="5"/>
     <row r="6" ht="16" customHeight="1" s="7">
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -570,7 +569,7 @@
           <t>We ran two independent analyses and required them to converge before accepting a result.
 ### Analysis A — genome-wide, phenotype-informed, hypothesis-free (primary)
 Exomiser 15.1.0 with the 2602 hg38 and 2602 phenotype data releases. Input was the unmodified proband
-VCF — 5,012,204 records, of which 4,740,790 carry the PASS filter (GRCh38, GATK 4.2.4.0) — together
+VCF — **5,012,204 records, of which 4,740,790 carry the PASS filter** (GRCh38, GATK 4.2.4.0) — together
 with the eight HPO terms extracted verbatim from the supplied clinical document:
 | HPO | Term |
 |---|---|
@@ -586,8 +585,8 @@
 child. We kept it because the clinical document states it and because it is informative for the mode
 of inheritance, but we flag it explicitly rather than let it pass as a proband phenotype.
 No gene panel, no candidate list and no reference to a disease name entered the configuration at any
-point. Prioritisation used hiPhivePrioritiser (human, mouse, fish and protein-interaction evidence)
-and omimPrioritiser. Inheritance models covered autosomal dominant, autosomal recessive
+point. Prioritisation used `hiPhivePrioritiser` (human, mouse, fish and protein-interaction evidence)
+and `omimPrioritiser`. Inheritance models covered autosomal dominant, autosomal recessive
 (homozygous and compound heterozygous), X-linked and mitochondrial. Frequency sources were UK10K and
 gnomAD exomes/genomes across five populations at a 2% maximum; pathogenicity sources were REVEL, MVP,
 AlphaMissense and SpliceAI.
@@ -595,51 +594,69 @@
 filter → 277,724 after the variant-effect filter → 11,255 after frequency → 9,935 after
 inheritance-mode compatibility, distributed across 3,139 genes.
 ### Result
-BUB1B ranked 2nd of 3,139 genes under the autosomal recessive model, and Exomiser assigned that
-ranking to ORPHA:1052, mosaic variegated aneuploidy syndrome — the correct disease, reached without
+**BUB1B ranked 2nd of 3,139 genes under the autosomal recessive model, and Exomiser assigned that
+ranking to ORPHA:1052, mosaic variegated aneuploidy syndrome** — the correct disease, reached without
 being told. Under the recessive model both variants were marked as contributing, so Exomiser
 reconstructed the compound heterozygous pair on its own.
 The same gene also took rank 1 under the autosomal dominant model, but that entry is an artefact we
-report rather than claim: Exomiser attached it to OMIM:114500, colorectal cancer (somatic), and
-it wins the top slot largely because the nonsense variant is on the ClinVar whitelist, which
-short-circuits variant scoring to 1.0. A single truncating allele in a recessive gene is not a
-dominant colorectal cancer diagnosis. The result we stand behind is rank 2, not rank 1. We say so
+report rather than claim: Exomiser attached it to **OMIM:114500, colorectal cancer (somatic)**, and
+it wins the top slot because a single truncating allele saturates the variant term of the dominant
+model. We originally wrote that the ClinVar whitelist was what short-circuited variant scoring to 1.0;
+**we tested that and it is wrong.** Planting an unclassified ClinVar nonsense record in the same gene
+(`chr15:40212550 G&gt;T`, no CLNSIG, not whitelisted) gives the identical variant score of 1.0000 — the
+`stop_gained` consequence alone saturates it (§ Benchmark, below). A single truncating allele in a
+recessive gene is not a dominant colorectal cancer diagnosis. **The result we stand behind is rank 2, not rank 1.** We say so
 because the honest reading of our own output matters more than the better-sounding headline.
 The combined score gap is real but moderate: 0.5871 (rank 1, AD) and 0.5538 (rank 2, AR) against
-0.2137 for the third-ranked gene — 2.59× the third gene for the recessive result we stand behind (2.75× for the dominant artefact), not an order of magnitude.
+0.2137 for the third-ranked gene — **2.59× the third gene for the recessive result we stand behind** (2.75× for the dominant artefact), not an order of magnitude.
 ### Robustness controls — including one that argues against us
-We ran twelve additional Exomiser analyses to test how much of the result comes from the phenotype
-and how much from the variant.
-Leave-one-HPO-out (8 runs). Removing each HPO term in turn: BUB1B remained rank 1 in all
-eight, with scores from 0.5447 to 0.7503. Removing the rhabdomyosarcoma term — the one a human
-would consider most diagnostic — actually raised the score to 0.7503. No single symptom carries the
+We ran twelve additional Exomiser analyses to test how much of the result comes from the phenotype and
+how much from the variant — eleven initially, plus one re-run after we found a flaw in our own control.
+**Leave-one-HPO-out (8 runs).** Removing each HPO term in turn: **BUB1B remained rank 1 in all
+eight**, with scores from 0.5447 to 0.7503. Removing the rhabdomyosarcoma term — the one a human
+would consider most diagnostic — actually *raised* the score to 0.7503. No single symptom carries the
 result.
-Unrelated HPO terms (2 runs, one of which corrects the other). Our first version of this control
+**Unrelated HPO terms (2 runs, one of which corrects the other).** Our first version of this control
 replaced the eight clinical terms with five we described as "clinically unrelated" — seizure
 (HP:0001250), hearing impairment (HP:0000365), atrial septal defect (HP:0001631), conjunctivitis
 (HP:0000509) and recurrent respiratory infections (HP:0002205). BUB1B came out rank 1, score 0.5506.
-That control was contaminated, and we caught it ourselves. Querying the HPO annotations for
-OMIM:257300 returns 59 terms, and two of our five are among them: seizure (HP:0001250, Nervous
+**That control was contaminated, and we caught it ourselves.** Querying the HPO annotations for
+OMIM:257300 returns 59 terms, and **two of our five are among them**: seizure (HP:0001250, Nervous
 System) and atrial septal defect (HP:0001631, Cardiovascular). Congenital heart defects including
 septal defects are an established feature of MVA, and BubR1 loss disrupts cardiac development
 (PMID 40055864). So the run was not a phenotype-free control at all — it fed the pipeline two genuine
 MVA features.
-We re-ran it with five terms verified against the same annotation set as absent from MVA1: hearing
+**We re-ran it with five terms verified against the same annotation set as absent from MVA1:** hearing
 impairment (HP:0000365), conjunctivitis (HP:0000509), recurrent respiratory infections (HP:0002205),
-headache (HP:0002315) and pruritus (HP:0000989). BUB1B still came out rank 1 of 4,565 genes, score
-0.4187. The conclusion survives a clean control.
-The comparison is itself informative. Removing the two contaminating terms drops the score from 0.5506
-to 0.4187 — about 24% — without changing the rank. That is the size of the phenotype's contribution
-here: measurable, and not enough to decide the answer. Script and log:
+headache (HP:0002315) and pruritus (HP:0000989). **BUB1B still came out top of the ranking, score 0.4187 on
+the dominant row.** The conclusion survives a clean control.
+*A note on the denominator, because we had this wrong.* An earlier version of this sentence said
+"rank 1 of 4,565 genes". 4,565 is the number of gene × inheritance-mode **rows** in that output file,
+not genes: the run covers **3,139 genes**, and of those only **257 receive a combined score above
+zero** (32 score ≥ 0.01) while the remaining rows are tied at the bottom rank with score 0. The
+honest denominator is 3,139 genes, of which 257 were scored at all.
+The comparison is informative, but we previously drew the wrong number from it. We wrote that
+removing the two contaminating terms drops the score from 0.5506 to 0.4187, "about 24%", and called
+that the size of the phenotype's contribution. **Both endpoints of that comparison are unrelated-HPO
+controls** — the contaminated one and its correction — so the delta measures what two leaked
+MVA-annotated terms were worth, not what the patient's phenotype is worth. **That figure is
+withdrawn.**
+The right comparison is the real phenotype against the clean control: **0.5871 with the patient's
+eight terms, 0.4187 with five verified-unrelated terms, Δ = 0.1684**, and both values reproduce to
+four decimal places when the same two alleles are planted into three unrelated healthy genomes
+(§ Benchmark). We do **not** convert that delta into a percentage of the score: Exomiser combines
+phenotype and variant evidence non-linearly, and 0.4187 is not a phenotype-free baseline, so a share
+is not defined. It is a sensitivity of the score to the HPO query. Script and log:
 `tools/control_hpo_r7.sh`, `tools/logs/controles_hpo_r7.log`.
-Least-specific term alone (1 run). With short stature (HP:0004322) as the only input, BUB1B fell
-to rank 4 and HK1 took the top slot.
-No phenotype at all (1 run). Exomiser terminates with an error; the tool requires at least one
+**Least-specific term alone (1 run).** With short stature (HP:0004322) as the only input, BUB1B fell
+to **rank 4** and HK1 took the top slot.
+**No phenotype at all (1 run).** Exomiser terminates with an error; the tool requires at least one
 HPO term, so this control could not be run.
-What this forces us to conclude. We cannot call this a phenotype-driven discovery. The signal
-comes from the variant — a ClinVar-whitelisted pathogenic nonsense allele in a constrained gene
-(LOEUF 0.588) — not from the phenotype. The accurate description is variant-driven and
-phenotype-consistent. What the phenotype does contribute is the choice between competing
+**What this forces us to conclude.** We cannot call this a phenotype-driven discovery. The signal
+comes from the **variant** — a pathogenic nonsense allele in a constrained gene (LOEUF 0.588) — not
+from the phenotype, and not from the database record either: with both ClinVar classifications
+stripped, the same molecular architecture still scores 0.5743 and still ranks first (§ Benchmark). The accurate description is **variant-driven and
+phenotype-consistent**. What the phenotype does contribute is the choice between competing
 interpretations of the same variant: it is the phenotype that makes Exomiser attach the recessive
 model to mosaic variegated aneuploidy rather than to somatic colorectal cancer, and the
 least-specific-term control shows the effect is real (one vague term is not enough to reach the top).
@@ -652,36 +669,36 @@
 ### Analysis B — targeted panel, orthogonal confirmation
 An 11-gene panel of MVA genes and phenocopies (BUB1B, CEP57, TRIP13, CENATAC, MAD1L1, MAD2L1BP,
 CEP192, BUB1, SMC5, TRIM37, CENPE) with 5 kb padding. Coordinates were retrieved programmatically
-from the Ensembl REST API (release 116) rather than from memory or a static file, and the
+from the **Ensembl REST API (release 116)** rather than from memory or a static file, and the
 provenance of every coordinate is recorded. The 1,532 PASS variants inside those intervals were
-annotated with the Ensembl VEP REST API and filtered for HIGH or MODERATE impact on the canonical
+annotated with the **Ensembl VEP REST API** and filtered for HIGH or MODERATE impact on the canonical
 transcript at gnomAD AF below 1% or absent.
 Exactly three variants survived. Two were in BUB1B; the third (MAD1L1 p.Arg59Cys) was a single allele
-in a recessive gene and cannot explain the phenotype. BUB1B was the only gene carrying two rare
-damaging alleles.
+in a recessive gene and cannot explain the phenotype. **BUB1B was the only gene carrying two rare
+damaging alleles.**
 ### Convergent answer
 | Variant | Consequence | gnomAD (max pop. AF) | ClinVar | Exomiser ACMG (AR model) |
 |---|---|---|---|---|
-| NM_001211.6:c.2210T&gt;G p.Leu737Ter | stop_gained | 9.98×10⁻⁵ (gnomAD exomes NFE) | 533901, Pathogenic/Likely pathogenic, 2★ | PATHOGENIC (PVS1, PM2_Supporting, PP4_Moderate, PP5_Strong) |
-| NM_001211.6:c.3006T&gt;G p.Asn1002Lys | missense | 8.99×10⁻⁷ (gnomAD exomes NFE) | not present | UNCERTAIN_SIGNIFICANCE (PM2_Supporting, PP4_Moderate, BP1) |
+| `NM_001211.6:c.2210T&gt;G` p.Leu737Ter | stop_gained | 9.98×10⁻⁵ (gnomAD exomes NFE) | 533901, Pathogenic/Likely pathogenic, 2★ | PATHOGENIC (PVS1, PM2_Supporting, PP4_Moderate, PP5_Strong) |
+| `NM_001211.6:c.3006T&gt;G` p.Asn1002Lys | missense | 8.99×10⁻⁷ (gnomAD exomes NFE) | not present | UNCERTAIN_SIGNIFICANCE (PM2_Supporting, PP4_Moderate, BP1) |
 Two notes on this table, both of which correct looser statements we could have made:
-- The two frequency sources disagree for the nonsense variant. Exomiser's bundled gnomAD gives
+- **The two frequency sources disagree for the nonsense variant.** Exomiser's bundled gnomAD gives
   9.98×10⁻⁵ (GNOMAD_E_NFE); the Ensembl VEP REST API returned ≈3×10⁻⁵ for the same variant. We report
   the Exomiser figure because it is the one the ranking was computed from, and we declare the
   discrepancy rather than pick the smaller number. Either way the allele is rare and there are no
   homozygotes.
-- The missense variant is not absent from gnomAD, as we first wrote. It is present at 8.99×10⁻⁷,
+- **The missense variant is not absent from gnomAD**, as we first wrote. It is present at 8.99×10⁻⁷,
   which is a single-observation-level frequency but not zero. It carries REVEL 0.472, MVP 0.852 and
   AlphaMissense 0.923 — the in-silico predictors disagree with each other, which is why we let it
   stand as a VUS rather than upgrade it.
-On ClinVar: c.3006T&gt;G is not in ClinVar. ClinVar contains c.3006T&gt;A
-(VCV004600147, NC_000015.10:40220611:T:A), a *different nucleotide substitution at the same
+On ClinVar: **c.3006T&gt;G is not in ClinVar.** ClinVar contains `c.3006T&gt;A`
+(VCV004600147, `NC_000015.10:40220611:T:A`), a *different nucleotide substitution at the same
 position* producing the same p.Asn1002Lys protein change, classified Uncertain significance —
-criteria provided, single submitter, last evaluated 2025-09-19. That classification does not
+criteria provided, single submitter, last evaluated 2025-09-19. That classification does **not**
 transfer: the two alleles differ in splicing potential and in mutational context, and a VUS
 transferred across alleles would in any case add no evidence. We did not use it.
-Diagnosis: mosaic variegated aneuploidy type 1 (MVA1, OMIM 257300), autosomal recessive, caused by
-compound heterozygosity in BUB1B. The truncating-plus-missense configuration matches the allelic
+**Interpretation: findings consistent with mosaic variegated aneuploidy type 1 (MVA1, OMIM 257300),
+autosomal recessive, through compound heterozygosity in BUB1B (phase not demonstrated; see limitations).** The truncating-plus-missense configuration matches the allelic
 pattern described in biallelic MVA patients — "in patients with biallelic mutations, a missense
 mutation pairs with a truncating mutation" (Suijkerbuijk 2010, PMID 20516114). Reading that pair as
 null-plus-hypomorph is our inference from the same work's observation of absent transcript from
@@ -694,31 +711,74 @@
 and chromosomal dosage from 10%-trimmed mean depth. Three of these are refinements of the same BAF
 statistic and only the dosage test is orthogonal — they are not four independent tests. Only the VCF
 was available, with no BAM, so no GC-LOESS normalisation was possible.
-We computed the detection limit instead of asserting a negative, and we state where the threshold
-comes from. Across the 22 autosomes at fixed depth (DP 40–48, 857,435 sites), the measured standard
-deviation of mean |BAF − 0.5| between chromosomes is 0.0035. Our 0.005 noise floor is therefore a
+**We computed the detection limit instead of asserting a negative, and we state where the threshold
+comes from.** Across the 22 autosomes at fixed depth (DP 40–48, 857,435 sites), the measured standard
+deviation of mean |BAF − 0.5| between chromosomes is **0.0035**. Our 0.005 noise floor is therefore a
 ≈1.4-SD criterion. Simulating mean |BAF − 0.5| at DP 44 against it, a clonal trisomy becomes
-detectable only when present in ~14% of cells.
+detectable only when present in **~14% of cells**.
 The conclusion does not depend on that choice, and every stricter choice hurts the assay rather than
-us: a conventional 2-SD criterion moves the limit to 16%, and 3-SD to 20%.
-Read sampling is not what sets that limit. The simulation subtracts the binomial baseline at
-DP 44, so the 0.005 threshold a signal must clear is the measured dispersion between chromosomes —
+us: a conventional 2-SD criterion moves the limit to **16%**, and 3-SD to **20%**.
+**Read sampling is not what sets that limit.** The simulation subtracts the binomial baseline at
+DP 44, so the 0.005 threshold a signal must clear is the *measured dispersion between chromosomes* —
 systematic library bias, not counting noise. The read-depth dosage test points the same way by a
 separate route: Poisson error when averaging a whole chromosome at 44× is ≈0.03%, orders of magnitude
 below the deviations observed. These are two different statistics and we do not conflate them; they
-agree on the conclusion that more sequencing depth would not move the limit.
+agree on the conclusion that **more sequencing depth would not move the limit**.
 Every candidate signal traced to coverage, segmental duplications (22q11, centromeres) or — partially
 — GC content. We flag that the GC explanation is incomplete: the measured GC–coverage correlation was
 r = 0.43 from a sparse sample, and chr21, the largest deviation, is GC-poor. Where dosage and BAF
 disagreed we favoured BAF, which is an internal per-site ratio and cancels coverage bias, and we
 report the dosage result as an open question.
-We therefore do not claim the child lacks mosaic aneuploidy — he has it by diagnostic definition.
+**We therefore do not claim the child lacks mosaic aneuploidy — he has it by diagnostic definition.**
 We claim this assay cannot resolve it. Variegation spreads the burden across chromosomes: an
 aneuploid fraction of ~30% distributed over the autosomes leaves each individual chromosome altered
-in roughly 1–2% of cells, which is 7–16× below the 14–16% detection limit. Bulk averaging erases
+in roughly **1–2% of cells, which is 7–16× below the 14–16% detection limit**. Bulk averaging erases
 variegation by construction, at any depth. Premature chromatid separation, the cytogenetic hallmark of MVA, leaves no trace in DNA
-sequence at all. The practical consequence is that aneuploidy burden is not a measurable endpoint
-in these data, which constrains any Track 2 proposal whose outcome depends on it.</t>
+sequence at all. The practical consequence is that **aneuploidy burden is not a measurable endpoint
+in these data**, which constrains any Track 2 proposal whose outcome depends on it.
+### Additional analysis — a pre-registered benchmark of this pipeline (MVA-Replay)
+Our controls above test one genome once. To find out what this pipeline does when the answer is
+*not* there, we built a benchmark on public data, **pre-registered it in git before running any case**
+(`replay/PREREGISTRO.md`, commit `8086dd4`, with three dated amendments), and sent the design — unrun
+— to two independent reviewers first. Their critique cut the design from ~150 runs to 61 and removed
+four ways in which it was rigged in our favour. No patient data is used anywhere in it: backgrounds
+are GIAB v4.2.1 benchmark genomes and 1000 Genomes 30× individuals; planted alleles are public ClinVar
+records; the analysis configuration is the one used above, frozen.
+**What score does a healthy genome produce under this phenotype?** Seven GIAB genomes, unspiked,
+queried with the patient's exact eight HPO terms, produce top-gene combined scores of 0.0578, 0.0599,
+0.2048, 0.4188, 0.4194, 0.4881 and **0.5619**. Our 0.5871 is above all seven, **by 0.025**. BUB1B does
+not appear in the ranked table of any of them. We state the direction of the bias: these callsets are
+autosome-only and high-confidence-region-only, retaining 6,510–9,486 variants against this patient's
+12,431 and ranking 1,872–2,495 genes against 3,139, so the comparison is conservative *in our favour*;
+and HG001 plus two trios is three independent units, not seven. A favourable null cleared by 0.025 is
+a narrow margin, not a separation.
+**Is the score a property of the patient's genome?** Planting the two public ClinVar records that
+reproduce this case's architecture (533901 `chr15:40209701 T&gt;G` nonsense, 4600147 `chr15:40220612 T&gt;A`
+VUS missense) into three unrelated healthy genomes returns **0.5871 with the real phenotype and
+0.4187 with five unrelated terms, identical to four decimal places in all three**. The gene reached
+the top position in 3/3 with the real phenotype and 2/3 with the unrelated one. The rank, not the
+score, is what the background changes.
+**How much of the score is the ClinVar record?** This is the result that went against what we had
+written. Holding gene, consequence, partner allele and phenotype fixed and changing only the ClinVar
+status:
+| Construct | Nonsense allele | Missense allele | Combined score |
+|---|---|---|---|
+| this case's architecture | ClinVar P/LP, whitelisted | ClinVar VUS | 0.5871 |
+| with the child's **real** missense (absent from ClinVar) | ClinVar P/LP | not in ClinVar | **0.5871** |
+| with an **unclassified** ClinVar nonsense | no CLNSIG, not whitelisted | ClinVar VUS | **0.5743** |
+| **with no ClinVar classification on either allele** | no CLNSIG | not in ClinVar | **0.5743** |
+Individual variant scores are identical in every row (1.0000 for the nonsense, 0.9229 for the
+missense). **Removing ClinVar entirely costs 0.0128 — 2.2% of the combined score — and does not
+change the top position in either background tested.** The whitelist adds `PP5_Strong` to the ACMG
+evidence; it is not what saturates the variant term, the `stop_gained` consequence is. An earlier
+draft of this report credited the ranking to the ClinVar whitelist; that attribution is corrected
+here. The finding is more robust than we had claimed: it would have been reached for a nonsense
+allele that no database had ever seen.
+**What the benchmark does not establish.** Every planted call is `PASS`, balanced and unambiguous, so
+this measures retrieval *given a perfect heterozygous call*, not end-to-end diagnostic sensitivity.
+Three case genes and one decoy are a replay of this case, not a general rare-disease benchmark. One
+of seven pre-registered predictions was contrary to its predicted direction and is reported as such
+in `replay/RESULTADOS.md`, together with the three conclusions of ours that the reviewers refuted.</t>
         </is>
       </c>
     </row>
@@ -910,12 +970,12 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>- Exomiser genome-wide run: 53 seconds wall clock (32-core CPU, 16 GB JVM heap).
-- Twelve robustness controls: about 10 minutes total.
+          <t>- Exomiser genome-wide run: **53 seconds** wall clock (32-core CPU, 16 GB JVM heap).
+- Twelve robustness controls: about 11 minutes total.
 - Targeted panel with REST annotation: under 5 minutes, dominated by API latency.
-- Mosaicism analysis: about 10 minutes of bcftools streaming.
+- Mosaicism analysis: about 10 minutes of `bcftools` streaming.
 - One-off setup: ≈55 GB of Exomiser reference data downloaded and extracted.
-- Marginal compute cost is effectively zero — a commodity workstation, no GPU, no cloud instance.
+- **Marginal compute cost is effectively zero** — a commodity workstation, no GPU, no cloud instance.
   Reproducing this on a laptop is realistic: only the 315 MB VCF and the phenotype document are
   needed, not the 85 GB of raw reads.</t>
         </is>
@@ -929,42 +989,40 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>We identified the causal variants through two independent analyses designed to check each other, and
-required them to converge before accepting a result.
-The primary analysis was deliberately hypothesis-free. Exomiser 15.1.0 (data release 2602, hg38) was
-run on the complete proband VCF — 4,740,790 PASS variants — driven only by the eight HPO terms taken
-verbatim from the clinical document. No gene panel, no candidate list and no mention of a disease
-name entered the configuration. Prioritisation combined hiPhive (human, mouse, fish and
-protein-interaction evidence) with the OMIM prioritiser across dominant, recessive, X-linked and
-mitochondrial models. BUB1B ranked 2nd of 3,139 genes under the recessive model, mapped by Exomiser
-to mosaic variegated aneuploidy syndrome (ORPHA:1052), with both variants flagged as contributing —
-the compound heterozygous pair reconstructed without instruction. The same gene took rank 1 under the
-dominant model, but attached to somatic colorectal cancer; we report that entry as an artefact of the
-ClinVar whitelist rather than claim it.
-The confirmatory analysis took the opposite approach: an 11-gene panel of MVA genes and phenocopies,
-coordinates fetched programmatically from the Ensembl REST API with provenance recorded, annotated
-through Ensembl VEP and filtered for HIGH/MODERATE impact below 1% gnomAD AF. Of 1,532 variants three
-survived; two were in BUB1B, the only gene carrying two rare damaging alleles.
-Both routes converge on NM_001211.6:c.2210T&gt;G p.Leu737Ter (nonsense; ClinVar 533901
-Pathogenic/Likely pathogenic; gnomAD 9.98×10⁻⁵) and c.3006T&gt;G p.Asn1002Lys (missense; gnomAD
-8.99×10⁻⁷; not in ClinVar), consistent with MVA1 (OMIM 257300) and with the truncating-plus-missense
-allelic pattern of viable MVA1.
-Twelve robustness controls, one of which argues against us. Leave-one-HPO-out keeps BUB1B at rank
-1 in all eight runs, so no single symptom drives the result — but substituting clinically unrelated
-HPO terms also returns BUB1B at rank 1. We therefore describe the finding as variant-driven and
-phenotype-consistent, not phenotype-driven: the ClinVar-whitelisted nonsense allele carries the
-ranking, and the phenotype's real contribution is selecting the recessive MVA interpretation over the
-dominant cancer artefact. Reporting this control costs us an argument; omitting it would have been
-the kind of thing a reviewer finds.
-We also asked whether mosaic aneuploidy is visible in the bulk WGS. It is not, and we computed why:
-simulating mean |BAF − 0.5| at DP 44 puts the detection limit at ~14% of cells for a clonal trisomy
-(16% under a stricter 2-SD criterion), while variegation leaves each chromosome at 1–2% of cells —
-7–16× below it. Aneuploidy burden is not a
-measurable endpoint in these data — a constraint that matters for evaluating any candidate therapy.
-Limitations. Phase cannot be established: no parental sample, and the variants lie ~11 kb apart,
-beyond read-backed phasing (confirmed by the absence of GATK phase tags on both). The functional
-consequence of p.Asn1002Lys is unproven, and its in-silico predictors disagree (REVEL 0.472,
-AlphaMissense 0.923). REMM and CADD were omitted. The genome-wide Exomiser run took 53 seconds on a commodity workstation with no GPU.</t>
+          <t>We identified the causal variants through two independent analyses required to converge.
+The primary analysis was hypothesis-free: Exomiser 15.1.0 (data 2602, hg38) on the complete proband
+VCF — 4,740,790 PASS variants — driven only by the eight HPO terms taken verbatim from the clinical
+document. No gene panel, no candidate list and no disease name entered the configuration.
+**BUB1B ranked 2nd of 3,139 genes under the recessive model, mapped by Exomiser to mosaic variegated
+aneuploidy syndrome (ORPHA:1052)**, both variants flagged as contributing. The same gene took rank 1
+under the dominant model but attached to somatic colorectal cancer; we report that as an artefact of
+a single truncating allele saturating the dominant model's variant term, not as a result.
+The confirmatory analysis was orthogonal: an 11-gene MVA panel, coordinates from the Ensembl REST API,
+annotated through VEP, filtered for HIGH/MODERATE impact below 1% gnomAD AF. Of 1,532 variants three
+survived; two were in BUB1B, the only gene with two rare damaging alleles.
+Both routes converge on **NM_001211.6:c.2210T&gt;G p.Leu737Ter** (nonsense; ClinVar 533901
+Pathogenic/Likely pathogenic; gnomAD 9.98×10⁻⁵) and **c.3006T&gt;G p.Asn1002Lys** (missense; gnomAD
+8.99×10⁻⁷; not in ClinVar) — the truncating-plus-missense allelic pattern of viable MVA1.
+**Twelve robustness controls, one of which argues against us.** Leave-one-HPO-out keeps BUB1B on top
+in all eight runs, but five verified-unrelated HPO terms also return it there (0.4187 against 0.5871).
+The finding is **variant-driven and phenotype-consistent**: the loss-of-function consequence carries
+the ranking; the phenotype selects the recessive MVA interpretation over the dominant artefact.
+**We then measured what this pipeline does when the answer is absent.** A benchmark pre-registered in
+git before any case ran — 61 runs, public data only, design critiqued by two independent reviewers —
+shows three things. Seven healthy GIAB genomes queried with the same eight terms produce top-gene
+scores of 0.058–0.562 against our 0.587, a margin of 0.025 on a null biased in our favour. Planting
+the same two public ClinVar alleles into three unrelated healthy genomes reproduces 0.5871 and 0.4187
+to four decimals — the score follows the alleles and the query, not the genome. And stripping both
+ClinVar classifications costs **0.0128, 2.2% of the score**, without changing the top position: the
+database record is not what drives the result, the truncating consequence is.
+Mosaic aneuploidy is not visible in the bulk WGS and we computed why: at DP 44 the detection limit is
+~14% of cells while variegation leaves each chromosome at 1–2%, 7–16× below it.
+**Limitations.** Phase is not observable here: no parental sample, no alignments (a VCF was
+distributed, so no read-backed phaser can run), 10,911 bp between the variants with no GATK phase tag,
+and neither they nor the only heterozygous site between them is in the 1000 Genomes 3,202-sample
+panel, so reference-panel phasing discards all three. Our pipeline is insensitive to phase in any
+case. The functional consequence of p.Asn1002Lys is unproven and its predictors disagree (REVEL 0.472,
+AlphaMissense 0.923). REMM and CADD were omitted. The genome-wide run took 53 seconds without a GPU.</t>
         </is>
       </c>
     </row>
@@ -1007,7 +1065,6 @@
     </row>
     <row r="3"/>
     <row r="4"/>
-    <row r="5"/>
     <row r="6" ht="16" customHeight="1" s="7">
       <c r="B6" s="1" t="inlineStr">
         <is>
@@ -1191,10 +1248,15 @@
 Cell lines derived from MVA patients with biallelic mutations show "an impaired mitotic checkpoint,
 chromosome alignment defects, and low overall BUBR1 abundance" (PMID 20516114), and allele-specific effects — not merely total BubR1 quantity — drive phenotypic
 heterogeneity (Sieben 2020, PMID 31738183).
-We were explicit about what we could not determine. Phase is not established: no parental
-samples, and the two variants lie ~11 kb apart, beyond read-backed phasing for short reads — a limit
-visible in the data itself, since GATK emitted no phase tags for either BUB1B variant while phasing
-three variants 5 bp apart elsewhere in the same VCF. Nonsense-mediated decay of the truncated
+We were explicit about what we could not determine. Phase is not established, and we measured that it is not
+establishable from these data: there are no parental samples, the challenge distributes a VCF with no
+alignments so no read-backed phaser can be run, and the two variants lie 10,911 bp apart with no GATK
+phase tag on either — a limit visible in the data itself, since GATK did phase three variants 5 bp
+apart elsewhere in the same VCF. Reference-panel phasing fails separately: all three heterozygous
+sites inside the interval are absent from the 1000 Genomes 3,202-sample phased panel, and Beagle 5.5
+drops all three. Our retrieval pipeline is insensitive to phase in any case: two pathogenic nonsense
+alleles declared in cis are still called compound heterozygous, still PATHOGENIC and still ranked
+first, at a 0.34% score penalty. Nonsense-mediated decay of the truncated
 transcript is unmeasured and we do not assert it either way without patient RNA. p.Asn1002Lys has
 no published functional assay, and its in-silico predictors disagree (REVEL 0.472, AlphaMissense
 0.923), which is why we let it stand as a VUS.
@@ -1248,24 +1310,23 @@
 increasing protein degradation and are correspondingly sensitive to proteasome inhibition; aneuploidy
 level was significantly associated with multiple myeloma patients' response to proteasome inhibitors
 (Ippolito 2024, PMID 39247952), on cohorts small enough (8 complete responders vs 50 progressive)
-that we treat it as motivation for an experiment, not prediction. The concentration reaches: EC50
+that we treat it as motivation, not prediction. The concentration reaches: EC50
 below 40 nM in highly aneuploid lines against a label Cmax of 89–120 ng/mL (231–312 nM) at
 1.3 mg/m² IV — a margin of 5.8–7.8× on total drug. The subcutaneous route does not pass once protein binding
 is considered, and we say so.
-It then fails filter four for this child, and we say so plainly: motor neuropathy in 8% of
-paediatric patients, on top of existing skeletal muscle atrophy. But filter four is patient-specific.
+It then fails filter four for this child: motor neuropathy in 8% of paediatric patients, on top of
+existing skeletal muscle atrophy. But filter four is patient-specific.
 For an MVA patient with an active malignancy — where the comparator is cytotoxic chemotherapy rather
 than nothing — the balance inverts, and biallelic BUB1B carries a high risk of embryonal tumours. Our
 deliverable is that answer prepared in advance, with its margin and its stopping rule.
-Strengths. Every candidate is killed or kept by a stated criterion, including our own preferred
-one. We report an antagonism a combination-minded team could walk into: reducing translation protects
+Strengths. Every candidate is killed or kept by a stated criterion, including our own. We report an antagonism a combination-minded team could walk into: reducing translation protects
 CIN cells from proteasome inhibition (PMID 31530568), so mTOR inhibitors would be predicted to
-antagonise rather than synergise. The five-filter framework transfers to any rare disease.
+antagonise rather than synergise. The framework transfers to any rare disease.
 Limitations. The proteasome dependency is established in cancer aneuploidy, not constitutional
 mosaicism; whether it transfers is precisely what our eight-week experiment tests, and we
-have not assumed it. The EC50 is a conservative bound read from a figure panel. Phase is unproven.
-And no disease-modifying drug can be recommended from these data today — the intervention that most
-changes his prognosis now is surveillance, not a molecule.</t>
+have not assumed it. The EC50 is a conservative bound read from a figure panel. Phase is unproven and, we show, unobservable in these data; parental genotyping is the cheapest experiment here.
+And no disease-modifying drug can be recommended from these data today — what most changes his
+prognosis now is surveillance, not a molecule.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Render the v4 pitch video, sync the methods form, trim both abstracts to 500 words
- video: slides re-rendered from slides.html, narration re-synthesised, 177.87 s measured by ffprobe
- methods_description_form_ciberpty.xlsx: every answer cell regenerated from the markdown; the
  Track 1 and Track 2 abstracts were 547 and 646 words against a 500-word limit and are now 484/489
- replay/mva_replay.py: fail early with the name of any missing resource instead of a bcftools
  error that reads like a missing allele
- submission LEEME reflects the regenerated PDFs

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Bin1pbSawAwvE2SkU7oJeK
</commit_message>
<xml_diff>
--- a/submission/methods_description_form_ciberpty.xlsx
+++ b/submission/methods_description_form_ciberpty.xlsx
@@ -569,7 +569,7 @@
           <t>We ran two independent analyses and required them to converge before accepting a result.
 ### Analysis A — genome-wide, phenotype-informed, hypothesis-free (primary)
 Exomiser 15.1.0 with the 2602 hg38 and 2602 phenotype data releases. Input was the unmodified proband
-VCF — **5,012,204 records, of which 4,740,790 carry the PASS filter** (GRCh38, GATK 4.2.4.0) — together
+VCF — 5,012,204 records, of which 4,740,790 carry the PASS filter (GRCh38, GATK 4.2.4.0) — together
 with the eight HPO terms extracted verbatim from the supplied clinical document:
 | HPO | Term |
 |---|---|
@@ -594,95 +594,120 @@
 filter → 277,724 after the variant-effect filter → 11,255 after frequency → 9,935 after
 inheritance-mode compatibility, distributed across 3,139 genes.
 ### Result
-**BUB1B is the top-ranked gene of the 3,139 in this run, and its recessive row is first of the 2,100
-recessive-model rows, mapped by Exomiser to ORPHA:1052, mosaic variegated aneuploidy syndrome** — the correct disease, reached without
+BUB1B is the top-ranked gene of the 3,139 in this run, and its recessive row is first of the 2,100
+recessive-model rows, mapped by Exomiser to ORPHA:1052, mosaic variegated aneuploidy syndrome — the correct disease, reached without
 being told. Under the recessive model both variants were marked as contributing, so Exomiser
 reconstructed the compound heterozygous pair on its own.
 The same gene also took rank 1 under the autosomal dominant model, but that entry is an artefact we
-report rather than claim: Exomiser attached it to **OMIM:114500, colorectal cancer (somatic)**, and
+report rather than claim: Exomiser attached it to OMIM:114500, colorectal cancer (somatic), and
 a single truncating allele saturates the variant term of the dominant model, which is why that row's
-score is 0.5871. **It is not why the dominant row outranks the recessive one**: in our benchmark the
+score is 0.5871. It is not why the dominant row outranks the recessive one: in our benchmark the
 dominant row wins for BUB1B in every construct tested, including one with two missense VUS and no
 truncating allele at all (0.1120 dominant against 0.0925 recessive). Exomiser's ordering prefers the
 dominant model here regardless of the allele architecture, and we report that rather than explain it.
 We also originally wrote that the ClinVar whitelist was what short-circuited variant scoring to 1.0;
-**we tested that and it is wrong.** Planting an unclassified ClinVar nonsense record in the same gene
+we tested that and it is wrong. Planting an unclassified ClinVar nonsense record in the same gene
 (`chr15:40212550 G&gt;T`, no CLNSIG, not whitelisted) gives the identical variant score of 1.0000 — the
 `stop_gained` consequence alone saturates it (§ Benchmark, below). A single truncating allele in a
-recessive gene is not a dominant colorectal cancer diagnosis. **The result we stand behind is rank 2, not rank 1.** We say so
+recessive gene is not a dominant colorectal cancer diagnosis. The result we stand behind is rank 2, not rank 1. We say so
 because the honest reading of our own output matters more than the better-sounding headline.
 *A note on what "rank 2" counts.* Exomiser's table lists one row per gene × inheritance mode. BUB1B
 occupies the first two rows: 0.5871 (dominant) and 0.5538 (recessive). The next row, 0.2137, belongs
-to FANCD2 — the **second gene**, not the third. So BUB1B is gene rank 1 of 3,139 and its recessive row
+to FANCD2 — the second gene, not the third. So BUB1B is gene rank 1 of 3,139 and its recessive row
 is rank 1 of 2,100 recessive rows; it sits second in the overall row ordering only because its own
-dominant row sits first. The combined score gap is real but moderate: **2.59× the next gene for the
-recessive result we stand behind** (2.75× for the dominant artefact), not an order of magnitude.
-**Stated plainly, because it is the honest reading of our own output.** The pipeline's top-ranked row
+dominant row sits first. The combined score gap is real but moderate: 2.59× the next gene for the
+recessive result we stand behind (2.75× for the dominant artefact), not an order of magnitude.
+Stated plainly, because it is the honest reading of our own output. The pipeline's top-ranked row
 for BUB1B is a *dominant* single-allele model, not the recessive compound-heterozygous model the
 diagnosis rests on — and our benchmark shows the dominant row wins for BUB1B in every construct we
 tested, including one with no truncating allele. The compound-heterozygous call is also invariant to
 phase: declaring both alleles on the same chromosome changes neither the call, nor the
-classification, nor the rank. **The recessive interpretation is supplied by the inheritance model of
-the disease and by the two-allele architecture, not by the ranking.** What the retrieval delivers is
+classification, nor the rank. The recessive interpretation is supplied by the inheritance model of
+the disease and by the two-allele architecture, not by the ranking. What the retrieval delivers is
 the right gene; the diagnosis is an interpretation we make on top of it, and we say so rather than
 let the leaderboard number imply otherwise.
 ### Robustness controls — including one that argues against us
-We ran twelve additional Exomiser analyses to test how much of the result comes from the phenotype and
-how much from the variant — eleven initially, plus one re-run after we found a flaw in our own control.
-**Leave-one-HPO-out (8 runs).** Removing each HPO term in turn: **BUB1B remained rank 1 in all
-eight**, with scores from 0.5447 to 0.7503. Removing the rhabdomyosarcoma term — the one a human
+We ran additional Exomiser analyses to test how much of the result comes from the phenotype and how
+much from the variant. We list them by family rather than by a single total, because the total has
+been miscounted in earlier drafts: eight leave-one-HPO-out runs, one least-specific-term-alone
+run, one shuffled-phenotype run, and the unrelated-HPO control, which we had to rebuild twice
+(original → r7 → r9). Output files for each are under `tools/results/controles/`.
+⚠️ Read this section together with the note at the end of it. The version of this control that
+travelled with our submitted entry is r7, and r7 was contaminated. The numbers below are the corrected
+r9 analysis. The submitted prediction CSV is unaffected and unchanged — it contains the two BUB1B
+variants and no control depends on it — so this is a correction to the write-up, not to the answer.
+Leave-one-HPO-out (8 runs). Removing each HPO term in turn: BUB1B remained rank 1 in all
+eight, with scores from 0.5447 to 0.7503. Removing the rhabdomyosarcoma term — the one a human
 would consider most diagnostic — actually *raised* the score to 0.7503. No single symptom carries the
 result.
-**Unrelated HPO terms (2 runs, one of which corrects the other).** Our first version of this control
+Unrelated HPO terms (three versions, each correcting the last). Our first version of this control
 replaced the eight clinical terms with five we described as "clinically unrelated" — seizure
 (HP:0001250), hearing impairment (HP:0000365), atrial septal defect (HP:0001631), conjunctivitis
 (HP:0000509) and recurrent respiratory infections (HP:0002205). BUB1B came out rank 1, score 0.5506.
-**That control was contaminated, and we caught it ourselves.** Querying the HPO annotations for
-OMIM:257300 returns 59 terms, and **two of our five are among them**: seizure (HP:0001250, Nervous
+That control was contaminated, and we caught it ourselves. Querying the HPO annotations for
+OMIM:257300 returns 59 terms, and two of our five are among them: seizure (HP:0001250, Nervous
 System) and atrial septal defect (HP:0001631, Cardiovascular). Congenital heart defects including
 septal defects are an established feature of MVA, and BubR1 loss disrupts cardiac development
 (PMID 40055864). So the run was not a phenotype-free control at all — it fed the pipeline two genuine
 MVA features.
-**We re-ran it with five terms verified against the same annotation set as absent from MVA1:** hearing
-impairment (HP:0000365), conjunctivitis (HP:0000509), recurrent respiratory infections (HP:0002205),
-headache (HP:0002315) and pruritus (HP:0000989). **BUB1B still came out top of the ranking, score 0.4187 on
-the dominant row.** The conclusion survives a clean control.
+We re-ran it (r7) with five terms verified as absent from MVA1: hearing impairment (HP:0000365),
+conjunctivitis (HP:0000509), recurrent respiratory infections (HP:0002205), headache (HP:0002315) and
+pruritus (HP:0000989). BUB1B came out rank 1, score 0.4187. This is the version that travelled
+with the submission, and it was contaminated too.
+The r7 check was against `OMIM:257300` and nothing else, which was not enough. Hearing impairment
+(HP:0000365) is annotated to OMIM:614114 (MVA2), to ORPHA:1052 (the MVA umbrella term) and
+directly to BUB1B, CEP57 and TRIP13. Exomiser scores phenotype similarity over the whole ontology
+graph, so a term annotated to *any* MVA disease leaks the answer back in. The same class of error,
+twice, from an incomplete verification.
+r9 — the clean control. Five terms checked programmatically against all four MVA identifiers *and*
+against the three MVA genes (`hpo/01_verificar.py`, result in `hpo/verificacion.json`): conjunctivitis
+(HP:0000509), recurrent respiratory infections (HP:0002205), headache (HP:0002315), pruritus
+(HP:0000989) and skin rash (HP:0000988), which replaces hearing impairment. BUB1B is still rank 1
+in the proband's genome, score 0.3965 on the dominant row. The conclusion survives a clean control;
+the score the submitted write-up quoted was inflated by 0.0222.
+Screening control terms by eye does not work, and we stopped doing it. Of thirteen candidate terms
+put through the automated check, four were rejected — three of them replacements we had proposed
+ourselves, because fever, dyspnoea and abdominal pain are each annotated to *TRIP13*.
+⚠️ What the rule still does not guarantee. It removes terms with a *direct* annotation. It does not
+remove terms that merely sit near an MVA term in the ontology graph, and Exomiser's similarity measure
+is graph-based. The defensible statement is *"no term in the control set is annotated to any MVA
+disease or MVA gene"*, not *"no term is related to MVA"*.
 *A note on the denominator, because we had this wrong.* An earlier version of this sentence said
-"rank 1 of 4,565 genes". 4,565 is the number of gene × inheritance-mode **rows** in that output file,
-not genes. The run covers **3,139 unique genes**; **257 of them have at least one row scoring above
-zero** and 32 have a row ≥ 0.01. Separately, and in the other unit, **4,262 of the 4,565 rows carry a
-score of zero** and are tied at the bottom rank. The honest denominator is 3,139 genes, of which 257
+"rank 1 of 4,565 genes". 4,565 is the number of gene × inheritance-mode rows in that output file,
+not genes. The run covers 3,139 unique genes; 257 of them have at least one row scoring above
+zero and 32 have a row ≥ 0.01. Separately, and in the other unit, 4,262 of the 4,565 rows carry a
+score of zero and are tied at the bottom rank. The honest denominator is 3,139 genes, of which 257
 were scored at all.
 The comparison is informative, but we previously drew the wrong number from it. We wrote that
 removing the two contaminating terms drops the score from 0.5506 to 0.4187, "about 24%", and called
-that the size of the phenotype's contribution. **Both endpoints of that comparison are unrelated-HPO
-controls** — the contaminated one and its correction — so the delta measures what two leaked
-MVA-annotated terms were worth, not what the patient's phenotype is worth. **That figure is
-withdrawn.**
-The right comparison is the real phenotype against the clean control: **0.5871 with the patient's
-eight terms, 0.4187 with five verified-unrelated terms, Δ = 0.1684**, and both values reproduce to
-four decimal places when the same two alleles are planted into three unrelated healthy genomes
-(§ Benchmark). We do **not** convert that delta into a percentage of the score: Exomiser combines
-phenotype and variant evidence non-linearly, and 0.4187 is not a phenotype-free baseline, so a share
-is not defined. It is a sensitivity of the score to the HPO query. Script and log:
-`tools/control_hpo_r7.sh`, `tools/logs/controles_hpo_r7.log`.
-**Least-specific term alone (1 run).** With short stature (HP:0004322) as the only input, BUB1B fell
-to **rank 4** and HK1 took the top slot.
-**No phenotype at all (1 run).** Exomiser terminates with an error; the tool requires at least one
+that the size of the phenotype's contribution. Both endpoints of that comparison are unrelated-HPO
+controls — the contaminated one and its correction — so the delta measures what two leaked
+MVA-annotated terms were worth, not what the patient's phenotype is worth. That figure is
+withdrawn.
+The right comparison is the real phenotype against the clean r9 control: 0.5871 with the
+patient's eight terms, 0.3965 with five verified-unrelated terms, Δ = 0.1906, and both values
+reproduce to four decimal places when the same two alleles are planted into three unrelated healthy
+genomes (§ Benchmark). We do not convert that delta into a percentage of the score: Exomiser
+combines phenotype and variant evidence non-linearly, and 0.3965 is not a phenotype-free baseline, so
+a share is not defined. It is a sensitivity of the score to the HPO query. Script:
+`tools/control_hpo_r9.sh`; per-run outputs in `tools/results/controles/`.
+Least-specific term alone (1 run). With short stature (HP:0004322) as the only input, BUB1B fell
+to rank 4 and HK1 took the top slot.
+No phenotype at all (1 run). Exomiser terminates with an error; the tool requires at least one
 HPO term, so this control could not be run.
-**What this forces us to conclude.** We cannot call this a phenotype-driven discovery. The signal
-comes from the **variant** — a pathogenic nonsense allele in a constrained gene (LOEUF 0.588) — not
+What this forces us to conclude. We cannot call this a phenotype-driven discovery. The signal
+comes from the variant — a pathogenic nonsense allele in a constrained gene (LOEUF 0.588) — not
 from the phenotype, and not from the database record either: with both ClinVar classifications
-stripped, the same molecular architecture still scores 0.5743 and still ranks first (§ Benchmark). The accurate description is **variant-driven and
-phenotype-consistent**. **And we removed the last positive role we had attributed to the phenotype, because we tested it and
-it was false.** We had written that the phenotype is what makes Exomiser attach the recessive model to
+stripped, the same molecular architecture still scores 0.5743 and still ranks first (§ Benchmark). The accurate description is variant-driven and
+phenotype-consistent. And we removed the last positive role we had attributed to the phenotype, because we tested it and
+it was false. We had written that the phenotype is what makes Exomiser attach the recessive model to
 mosaic variegated aneuploidy rather than to somatic colorectal cancer. Re-running the clean
 unrelated-HPO control with variant-level output shows the same two mappings — recessive row →
 *Mosaic variegated aneuploidy syndrome*, dominant row → *Colorectal cancer, somatic* — under five
 clinically unrelated terms. The disease assignment comes from the gene's known inheritance modes via
 the OMIM prioritiser, not from the phenotype.
-What the phenotype measurably does in this case is move the combined score by 0.1684 without changing
-the top position. The least-specific-term control shows it is not nothing (short stature alone drops
+What the phenotype measurably does in this case is move the combined score by 0.1906 without changing
+the top position in the proband's genome. The least-specific-term control shows it is not nothing (short stature alone drops
 BUB1B to rank 4), but it does not select the interpretation, it does not choose the disease mapping,
 and it does not decide the answer.
 That is a narrower claim than "our pipeline found it from the symptoms", and it is the one the data
@@ -694,36 +719,36 @@
 ### Analysis B — targeted panel, orthogonal confirmation
 An 11-gene panel of MVA genes and phenocopies (BUB1B, CEP57, TRIP13, CENATAC, MAD1L1, MAD2L1BP,
 CEP192, BUB1, SMC5, TRIM37, CENPE) with 5 kb padding. Coordinates were retrieved programmatically
-from the **Ensembl REST API (release 116)** rather than from memory or a static file, and the
+from the Ensembl REST API (release 116) rather than from memory or a static file, and the
 provenance of every coordinate is recorded. The 1,532 PASS variants inside those intervals were
-annotated with the **Ensembl VEP REST API** and filtered for HIGH or MODERATE impact on the canonical
+annotated with the Ensembl VEP REST API and filtered for HIGH or MODERATE impact on the canonical
 transcript at gnomAD AF below 1% or absent.
 Exactly three variants survived. Two were in BUB1B; the third (MAD1L1 p.Arg59Cys) was a single allele
-in a recessive gene and cannot explain the phenotype. **BUB1B was the only gene carrying two rare
-damaging alleles.**
+in a recessive gene and cannot explain the phenotype. BUB1B was the only gene carrying two rare
+damaging alleles.
 ### Convergent answer
 | Variant | Consequence | gnomAD (max pop. AF) | ClinVar | Exomiser ACMG (AR model) |
 |---|---|---|---|---|
 | `NM_001211.6:c.2210T&gt;G` p.Leu737Ter | stop_gained | 9.98×10⁻⁵ (gnomAD exomes NFE) | 533901, Pathogenic/Likely pathogenic, 2★ | PATHOGENIC (PVS1, PM2_Supporting, PP4_Moderate, PP5_Strong) |
 | `NM_001211.6:c.3006T&gt;G` p.Asn1002Lys | missense | 8.99×10⁻⁷ (gnomAD exomes NFE) | not present | UNCERTAIN_SIGNIFICANCE (PM2_Supporting, PP4_Moderate, BP1) |
 Two notes on this table, both of which correct looser statements we could have made:
-- **The two frequency sources disagree for the nonsense variant.** Exomiser's bundled gnomAD gives
+- The two frequency sources disagree for the nonsense variant. Exomiser's bundled gnomAD gives
   9.98×10⁻⁵ (GNOMAD_E_NFE); the Ensembl VEP REST API returned ≈3×10⁻⁵ for the same variant. We report
   the Exomiser figure because it is the one the ranking was computed from, and we declare the
   discrepancy rather than pick the smaller number. Either way the allele is rare and there are no
   homozygotes.
-- **The missense variant is not absent from gnomAD**, as we first wrote. It is present at 8.99×10⁻⁷,
+- The missense variant is not absent from gnomAD, as we first wrote. It is present at 8.99×10⁻⁷,
   which is a single-observation-level frequency but not zero. It carries REVEL 0.472, MVP 0.852 and
   AlphaMissense 0.923 — the in-silico predictors disagree with each other, which is why we let it
   stand as a VUS rather than upgrade it.
-On ClinVar: **c.3006T&gt;G is not in ClinVar.** ClinVar contains `c.3006T&gt;A`
+On ClinVar: c.3006T&gt;G is not in ClinVar. ClinVar contains `c.3006T&gt;A`
 (VCV004600147, canonical SPDI `NC_000015.10:40220611:T:A`, 0-based, corresponding to VCF position 40220612), a *different nucleotide substitution at the same
 position* producing the same p.Asn1002Lys protein change, classified Uncertain significance —
-criteria provided, single submitter, last evaluated 2025-09-19. That classification does **not**
+criteria provided, single submitter, last evaluated 2025-09-19. That classification does not
 transfer: the two alleles differ in splicing potential and in mutational context, and a VUS
 transferred across alleles would in any case add no evidence. We did not use it.
-**Interpretation: findings consistent with mosaic variegated aneuploidy type 1 (MVA1, OMIM 257300),
-autosomal recessive, through compound heterozygosity in BUB1B (phase not demonstrated; see limitations).** The truncating-plus-missense configuration matches the allelic
+Interpretation: findings consistent with mosaic variegated aneuploidy type 1 (MVA1, OMIM 257300),
+autosomal recessive, through compound heterozygosity in BUB1B (phase not demonstrated; see limitations). The truncating-plus-missense configuration matches the allelic
 pattern described in biallelic MVA patients — "in patients with biallelic mutations, a missense
 mutation pairs with a truncating mutation" (Suijkerbuijk 2010, PMID 20516114). Reading that pair as
 null-plus-hypomorph is our inference from the same work's observation of absent transcript from
@@ -736,88 +761,124 @@
 and chromosomal dosage from 10%-trimmed mean depth. Three of these are refinements of the same BAF
 statistic and only the dosage test is orthogonal — they are not four independent tests. Only the VCF
 was available, with no BAM, so no GC-LOESS normalisation was possible.
-**We computed the detection limit instead of asserting a negative, and we state where the threshold
-comes from.** Across the 22 autosomes at fixed depth (DP 40–48, 857,435 sites), the measured standard
-deviation of mean |BAF − 0.5| between chromosomes is **0.0035**. Our 0.005 noise floor is therefore a
+We computed the detection limit instead of asserting a negative, and we state where the threshold
+comes from. Across the 22 autosomes at fixed depth (DP 40–48, 857,435 sites), the measured standard
+deviation of mean |BAF − 0.5| between chromosomes is 0.0035. Our 0.005 noise floor is therefore a
 ≈1.4-SD criterion. Simulating mean |BAF − 0.5| at DP 44 against it, a clonal trisomy becomes
-detectable only when present in **~14% of cells**.
+detectable only when present in ~14% of cells.
 The conclusion does not depend on that choice, and every stricter choice hurts the assay rather than
-us: a conventional 2-SD criterion moves the limit to **16%**, and 3-SD to **20%**.
-**Read sampling is not what sets that limit.** The simulation subtracts the binomial baseline at
+us: a conventional 2-SD criterion moves the limit to 16%, and 3-SD to 20%.
+Read sampling is not what sets that limit. The simulation subtracts the binomial baseline at
 DP 44, so the 0.005 threshold a signal must clear is the *measured dispersion between chromosomes* —
 systematic library bias, not counting noise. The read-depth dosage test points the same way by a
 separate route: Poisson error when averaging a whole chromosome at 44× is ≈0.03%, orders of magnitude
 below the deviations observed. These are two different statistics and we do not conflate them; they
-agree on the conclusion that **more sequencing depth would not move the limit**.
+agree on the conclusion that more sequencing depth would not move the limit.
 Every candidate signal traced to coverage, segmental duplications (22q11, centromeres) or — partially
 — GC content. We flag that the GC explanation is incomplete: the measured GC–coverage correlation was
 r = 0.43 from a sparse sample, and chr21, the largest deviation, is GC-poor. Where dosage and BAF
 disagreed we favoured BAF, which is an internal per-site ratio and cancels coverage bias, and we
 report the dosage result as an open question.
-**We therefore do not claim the child lacks mosaic aneuploidy — he has it by diagnostic definition.**
+We therefore do not claim the child lacks mosaic aneuploidy — he has it by diagnostic definition.
 We claim this assay cannot resolve it. Variegation spreads the burden across chromosomes: an
 aneuploid fraction of ~30% distributed over the autosomes leaves each individual chromosome altered
-in roughly **1–2% of cells, which is 7–16× below the 14–16% detection limit**. Bulk averaging erases
+in roughly 1–2% of cells, which is 7–16× below the 14–16% detection limit. Bulk averaging erases
 variegation by construction, at any depth. Premature chromatid separation, the cytogenetic hallmark of MVA, leaves no trace in DNA
-sequence at all. The practical consequence is that **aneuploidy burden is not a measurable endpoint
-in these data**, which constrains any Track 2 proposal whose outcome depends on it.
+sequence at all. The practical consequence is that aneuploidy burden is not a measurable endpoint
+in these data, which constrains any Track 2 proposal whose outcome depends on it.
 ### Additional analysis — a pre-registered benchmark of this pipeline (MVA-Replay)
 Our controls above test one genome once. To find out what this pipeline does when the answer is
-*not* there, we built a benchmark on public data, **pre-registered it in git before running any case**
+*not* there, we built a benchmark on public data, pre-registered it in git before running any case
 (`replay/PREREGISTRO.md`, commit `8086dd4`, with three dated amendments), and sent the design — unrun
 — to two independent reviewers first. Their critique cut the design from ~150 runs to 61 and removed
 four ways in which it was rigged in our favour. No patient data is used anywhere in it: backgrounds
 are GIAB v4.2.1 benchmark genomes and 1000 Genomes 30× individuals; planted alleles are public ClinVar
 records; the analysis configuration is the one used above, frozen.
-**What score does a healthy genome produce under this phenotype?** Seven GIAB genomes, unspiked,
+What score does a healthy genome produce under this phenotype? Seven GIAB genomes, unspiked,
 queried with the patient's exact eight HPO terms, produce top-gene combined scores of 0.0578, 0.0599,
-0.2048, 0.4188, 0.4194, 0.4881 and **0.5619**. Our 0.5871 is above all seven, **by 0.025**. BUB1B does
+0.2048, 0.4188, 0.4194, 0.4881 and 0.5619. Our 0.5871 is above all seven, by 0.025. BUB1B does
 not appear in the ranked table of any of them. We state the direction of the bias: these callsets are
-autosome-only and high-confidence-region-only, retaining **5,079–6,912 unique variants against this
-patient's 8,939** and ranking 1,872–2,495 genes against 3,139, so the comparison is conservative *in
+autosome-only and high-confidence-region-only, retaining 5,079–6,912 unique variants against this
+patient's 8,939 and ranking 1,872–2,495 genes against 3,139, so the comparison is conservative *in
 our favour*;
 and HG001 plus two trios is three independent units, not seven. A favourable null cleared by 0.025 is
 a narrow margin, not a separation.
-**Is the score a property of the patient's genome?** Planting the two public ClinVar records that
+Is the score a property of the patient's genome? Planting the two public ClinVar records that
 reproduce this case's architecture (533901 `chr15:40209701 T&gt;G` nonsense, 4600147 `chr15:40220612 T&gt;A`
-VUS missense) into three unrelated healthy genomes returns **0.5871 with the real phenotype and
-0.4187 with five unrelated terms, identical to four decimal places in all three**. The gene reached
-the top position in 3/3 with the real phenotype and 2/3 with the unrelated one. The rank, not the
-score, is what the background changes.
-**How much of the score is the ClinVar record?** This is the result that went against what we had
+VUS missense) into three unrelated healthy genomes returns 0.5871 with the real phenotype and
+0.3965 with the five clean r9 unrelated terms, identical to four decimal places in all three. The narrow
+statement is the one `replay/RESULTADOS.md` §2 makes: under this frozen pipeline, and given that none
+of the three backgrounds carries a retained BUB1B variant of its own, the planted gene's combined score
+does not move with the background while its rank does. That is stability of the score across the
+backgrounds we tested — one deterministic computation run three times — not a demonstration that the
+score is independent of the genome in general. A background carrying its own BUB1B variant (the
+1000 Genomes tier shows one, HG00101) was not tested with planted alleles, and our phase pilot already
+shows the score is not fully determined by the two alleles (0.9339 *cis* vs 0.9305 *trans*, § Phase).
+| Background | Real HPO, rank | Clean unrelated HPO, rank | Top gene under unrelated HPO |
+|---|---|---|---|
+| HG001 | 1 | 1 | BUB1B 0.3965 |
+| HG002 | 1 | 2 | KRT17 0.5766 |
+| HG005 | 1 | 3 | TNF 0.7436 |
+So with the real phenotype BUB1B is first in 3 of 3; with a clean unrelated phenotype it is first in
+1 of 3. Under the contaminated r7 set the same cells read 1 / 1 / 3, so the correction moves
+exactly one background, HG002. Neither KRT17 nor TNF is directly annotated to any of the five control
+terms — we checked `genes_to_phenotype.txt` — so the displacement is Exomiser's graph-based semantic
+similarity, and the replacement term "skin rash" sits near KRT17's cutaneous disease terms. In the
+proband's own genome BUB1B remains rank 1 under the clean control.
+How much of the score is the ClinVar record? This is the result that went against what we had
 written. Holding gene, consequence, partner allele and phenotype fixed and changing only the ClinVar
 status:
 | Construct | Nonsense allele | Missense allele | Combined score |
 |---|---|---|---|
 | this case's architecture | ClinVar P/LP, whitelisted | ClinVar VUS | 0.5871 |
-| with the child's **real** missense (absent from ClinVar) | ClinVar P/LP | not in ClinVar | **0.5871** |
-| with an **unclassified** ClinVar nonsense | no CLNSIG, not whitelisted | ClinVar VUS | **0.5743** |
-| **with no ClinVar classification on either allele** | no CLNSIG | not in ClinVar | **0.5743** |
+| with the child's real missense (absent from ClinVar) | ClinVar P/LP | not in ClinVar | 0.5871 |
+| with an unclassified ClinVar nonsense | no CLNSIG, not whitelisted | ClinVar VUS | 0.5743 |
+| with no ClinVar classification on either allele | no CLNSIG | not in ClinVar | 0.5743 |
 Individual variant scores are identical in every row (1.0000 for the nonsense, 0.9229 for the
-missense). **The combined score falls by 0.0128 and the top position does not change in either background
-tested; Exomiser's own call moves from PATHOGENIC to LIKELY_PATHOGENIC.** We do not express 0.0128 as
+missense). The combined score falls by 0.0128 and the top position does not change in either background
+tested; Exomiser's own call moves from PATHOGENIC to LIKELY_PATHOGENIC. We do not express 0.0128 as
 a percentage of the score, for the same reason we withdrew the phenotype percentage above: the
 combination is non-linear and a share is not defined.
-**What this does and does not establish.** We could not delete ClinVar's record for the child's own
+What this does and does not establish. We could not delete ClinVar's record for the child's own
 allele, so the last two rows substitute a *different* `stop_gained` at `chr15:40212550` — a ClinVar
 record carrying no classification and no whitelist flag. Gene, consequence class, partner allele and
 phenotype are held fixed; the locus is not. It therefore refutes our earlier claim that ClinVar
 whitelisting is what saturates the variant term — an unclassified nonsense reaches the same 1.0000 —
 and it shows the top position survives without any ClinVar classification in these two backgrounds. It
-does **not** show that an allele no database had ever recorded would rank identically, and it is not a
+does not show that an allele no database had ever recorded would rank identically, and it is not a
 deletion of ClinVar from this case's own variant.
-**The principal null experiment is still open.** The pre-registered design calls for 37 healthy
-genomes; the seven GIAB genomes above are complete and the 30 unrelated 1000 Genomes genomes are still
-running at the time of writing. The prediction is stated against the **maximum**, so a single
-exceedance falsifies it, and the sentences we will publish for each outcome were frozen before those
-runs finished (`replay/RESULTADOS.md` §8).
-**What the benchmark does not establish.** Every planted call is `PASS`, balanced and unambiguous, so
+The principal null experiment has now finished. The pre-registered design calls for 37 healthy
+genomes. The seven GIAB genomes are above; the 30 unrelated 1000 Genomes genomes are complete, with
+a maximum top-gene combined score of 0.5207 (CDH1, HG01885) and 0 of 30 exceeding 0.5871. The
+prediction was stated against the maximum, so a single exceedance would have falsified it, and the
+sentence published for this outcome was frozen before any of those runs finished
+(`replay/RESULTADOS.md` §8). Effective independence is roughly 33 unrelated individuals plus two trios,
+not 37 draws, and both callsets carry a lower rare-variant burden than clinical WGS, which lowers
+healthy top scores and biases the comparison *in our favour*.
+⚠️ One qualifier: *"BUB1B does not appear in the ranked table"* holds for the seven GIAB genomes. In
+the 1000 Genomes tier BUB1B does appear once, in HG00101, at rank 138 with a score of 0.0002. P-A2 was
+stated as "absent or below 0.25", so it holds — but the stronger wording does not.
+Pre-registered predictions, re-scored against each definition. The corrected control changes one
+of them, and it changes it against us, which is the outcome we pre-committed to publishing:
+| Prediction, as locked | Status |
+|---|---|
+| P-A — 0.5871 above every healthy genome's top score | confirmed (0 of 7 GIAB and 0 of 30 1000G exceed it) |
+| P-A2 — BUB1B absent or &lt; 0.25 in healthy genomes | confirmed (absent in 7/7 GIAB; 0.0002 in one 1000G genome) |
+| P-B1 — planted BUB1B rank 1 in 3/3 with real HPO | confirmed |
+| P-B2 — planted BUB1B rank 1 in ≥ 2/3 with unrelated HPO | falsified with the clean control (1/3). It read confirmed (2/3) only with the contaminated set |
+| P-B3 — planted decoy rank 1 in ≥ 2/3 with real HPO | not evaluable as locked — a pool defect our own ingestion check caught; the corrected construct ran contrary to the predicted direction |
+| P-B4 — Δ(real − unrelated) &lt; 0.20 | confirmed (0.1906 with the clean control, against 0.1684 with the contaminated one); the percentage form is withdrawn |
+| P-C — monotonic gradient, C-hi − C-lo ≥ 0.10 | confirmed (0.8212) — our causal reading of it is retracted |
+That is five confirmed, one falsified and one not evaluable. The falsification is P-B2, and the
+pre-registration said in advance that we *expected our own pipeline to fail this one* and pre-committed
+to publishing it if it did (`replay/PREREGISTRO.md`). We are not presenting it as a victory; we are
+presenting it because we said we would.
+What the benchmark does not establish. Every planted call is `PASS`, balanced and unambiguous, so
 this measures retrieval *given a perfect heterozygous call*, not end-to-end diagnostic sensitivity.
-Three case genes and one decoy are a replay of this case, not a general rare-disease benchmark. Of
-seven pre-registered predictions, five are confirmed, one is still open and one was not evaluable in
-its locked form because of a pool defect our own ingestion check caught; in the corrected construct it
-ran contrary to the predicted direction. All of this, and the three conclusions of ours that the
-reviewers refuted, is in `replay/RESULTADOS.md`.</t>
+Three case genes and one decoy are a replay of this case, not a general rare-disease benchmark. Thirty
+seven healthy genomes are not a validation cohort, and the GIAB and 1000 Genomes callsets share biases
+of their own. All of this, and the three conclusions of ours that the reviewers refuted, is in
+`replay/RESULTADOS.md`.</t>
         </is>
       </c>
     </row>
@@ -835,16 +896,16 @@
 - OpenAI, Codex (gpt-5.6), Plus plan, "Improve the model for everyone" disabled.
 - xAI Grok 4.6 via Cursor, Pro plan, Privacy Mode enabled (zero data retention at Cursor
   and at the underlying model providers).
-- Piper TTS (en_US-ryan-high) — open-source, run entirely on local hardware with no cloud
+- Piper TTS (`en_US-ryan-high`) — open-source, run entirely on local hardware with no cloud
   service and no API key. Used only to narrate the pitch video. Listed for completeness; it is not a
   commercial service.
 How these tools were used, and how they were not. The language models were used for literature
 retrieval and citation checking, for adversarial review of our own drafts, and for writing. They were
 also used against us on purpose: two independent models were asked to attack our reports, and the
 corrections they produced — including a claim of ours that contradicted our own data file — are
-recorded in the repository under evidencia/.
+recorded in the repository under `evidencia/`.
 No block of the VCF and no genotype table was ever sent to a language model. All genomic work ran
-on local tools (bcftools, Exomiser 15.1.0) and on annotation APIs — Ensembl VEP and ClinVar — that
+on local tools (`bcftools`, Exomiser 15.1.0) and on annotation APIs — Ensembl VEP and ClinVar — that
 the hackathon policy names explicitly as acceptable. What the models saw were named variants, HPO
 terms and reasoning: exactly the category the policy classifies as a "finding" and permits retaining.</t>
         </is>
@@ -874,10 +935,10 @@
       <c r="B12" s="3" t="inlineStr">
         <is>
           <t>Manual review was limited to two decisions, both documented:
-1. **Confirming the compound-heterozygous pair.** Both analyses proposed the pair automatically; we
+1. Confirming the compound-heterozygous pair. Both analyses proposed the pair automatically; we
    verified the genotypes (0/1 for both), read depths (46× and 28×) and allelic balance
    (21,25 and 15,13) directly in the VCF.
-2. **Adjudicating two secondary candidates** (see Q10).
+2. Adjudicating two secondary candidates (see Q10).
 No variant was added, removed or re-scored, and no gene was moved in the ranking. There is one
 interpretive judgement, made in the open: Exomiser emitted both a dominant and a recessive row for
 BUB1B and scored the dominant one higher, and we report the recessive one as the result because the
@@ -913,9 +974,9 @@
 - Exomiser 15.1.0 with data releases 2602_hg38 and 2602_phenotype
 - gnomAD v4 (via Exomiser and VEP)
 - ClinVar, GRCh38 (NCBI FTP snapshot and E-utilities)
-- Human Phenotype Ontology (hp.obo, genes_to_phenotype.txt)
+- Human Phenotype Ontology (`hp.obo`, `genes_to_phenotype.txt`)
 - REVEL, MVP, AlphaMissense and SpliceAI (via the Exomiser bundle)
-- OMIM and Orphanet identifiers via the Exomiser omimPrioritiser
+- OMIM and Orphanet identifiers via the Exomiser `omimPrioritiser`
 - Published literature (PubMed / Europe PMC), cited by PMID</t>
         </is>
       </c>
@@ -940,19 +1001,43 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Yes, and it did so without being told to. Exomiser's AUTOSOMAL_RECESSIVE_COMP_HET mode flagged both
+          <t>Yes, and it did so without being told to. Exomiser's `AUTOSOMAL_RECESSIVE_COMP_HET` mode flagged both
 BUB1B variants as contributing under the recessive model. The targeted analysis independently
 selected any gene carrying two rare damaging alleles, which returned BUB1B alone.
-Neither method can establish phase, and the data show why. There is no parental sample, and the
-two variants lie ~11 kb apart, far beyond read-backed phasing range for Illumina paired-end reads.
-This is not a theoretical limit in this VCF: GATK emitted no PGT/PID phasing tags for either
-BUB1B variant, while it did phase three FANCD2 variants spanning 5 bp into a single haplotype
-(PID=10046720_C_T) elsewhere in the same file. Read-backed phasing worked where the physical
-distance allowed it and was silent where it did not.
+Neither method can establish phase, and we went and measured why rather than asserting it.
+*Read-backed phasing is closed by what the challenge distributes.* There is no parental sample, and
+the dataset is a VCF with no BAM or CRAM, so no read-backed phaser (WhatsHap, HapCUT2) can be run at
+all. What the VCF shows is consistent: GATK emitted no `PGT`/`PID` tags for either BUB1B variant,
+which sit 10,911 bp apart, while it *did* phase three FANCD2 variants spanning 5 bp into a single
+haplotype (`PID=10046720_C_T`) elsewhere in the same file. Physical phasing worked where the distance
+allowed it and was silent where it did not.
+*Reference-panel phasing is closed by the panel.* Inside the 10,911 bp interval the patient carries
+exactly three heterozygous sites — the two causal variants and `chr15:40216470 A&gt;G` — and all three
+are absent from the 1000 Genomes 30× GRCh38 phased panel (3,202 individuals, 6,404 haplotypes). The
+nearest panel-present heterozygous markers are 16.8 kb upstream (AF 0.0016) and 809 bp downstream
+(AF 0.0075), with nothing in between that could link the two alleles. Beagle 5.5 run against that
+panel confirms it operationally: 1,391 of the patient's 1,452 window variants survive, and all three
+of the sites that matter are dropped, because a reference-panel phaser emits the panel's markers. The
+absence is what the frequencies predict — expected copy counts in 6,404 haplotypes are 0.64 for the
+nonsense (gnomAD max AF 1.0 × 10⁻⁴) and 0.006 for the missense (9.0 × 10⁻⁷); reaching a 95%
+chance of observing the missense would need on the order of 3 × 10⁶ haplotypes.
+*And our own pipeline would not have used phase if we had it.* In a controlled test on public data,
+Exomiser reads phase into its ACMG evidence (trans → PM3, cis → BP2) but not into the
+compound-heterozygous model: two pathogenic nonsense alleles declared on the same chromosome are
+still called AR_COMP_HET, both still marked contributing, still classified PATHOGENIC, and still
+ranked first. The combined score moves by 0.0034 in absolute terms (trans 0.9339, cis 0.9305,
+unphased 0.9325) — an absolute difference, not a share.
 The compound-heterozygous interpretation therefore rests on allele rarity, the known recessive
 inheritance of MVA1, the phenotype match, and the absence of homozygotes in gnomAD — not on a
-demonstrated trans configuration. Parental testing would settle it, and it is the single
-highest-value follow-up experiment for this case.</t>
+demonstrated *trans* configuration, which is not observable in these data. Parental genotyping at
+the two loci is the single highest-value follow-up for this case; long-read or linked-read
+sequencing of the child, or allele-specific analysis of the BUB1B transcript, would also settle it.
+All three require new laboratory work.
+⚠️ Settling phase would not settle the missense. A confirmed *trans* configuration supports the
+compound-heterozygous model and contributes PM3-type evidence; it does not on its own reclassify
+p.Asn1002Lys from uncertain significance. Function is a separate question and would need a functional
+assay. The *cis* result is the decisive one in the other direction: it would refute this
+interpretation.</t>
         </is>
       </c>
     </row>
@@ -968,11 +1053,11 @@
 which carry an ACMG classification. Three unique variants reached pathogenic or likely pathogenic
 (four rows — the BUB1B nonsense appears twice, once under the AD model and once under the AR model).
 Two of the three lie outside BUB1B, and both were adjudicated as non-reportable:
-FANCD2 chr3:10046723 AG&gt;A — ENST00000675286.1:c.1278+1del, Exomiser ACMG PATHOGENIC. Three
+FANCD2 chr3:10046723 `AG&gt;A` — `ENST00000675286.1:c.1278+1del`, Exomiser ACMG PATHOGENIC. Three
 independent reasons not to report it, in order of weight:
 1. The variant is not isolated: three co-phased changes in one splice region. GATK phased it
-   onto a single haplotype (PID=10046720_C_T) with two neighbours within 6 bp — chr3:10046720
-   C&gt;T, chr3:10046723 AG&gt;A and chr3:10046725 TAAG&gt;T (c.1278+3_1278+5del). All three sit at an
+   onto a single haplotype (`PID=10046720_C_T`) with two neighbours within 6 bp — chr3:10046720
+   `C&gt;T`, chr3:10046723 `AG&gt;A` and chr3:10046725 `TAAG&gt;T` (`c.1278+3_1278+5del`). All three sit at an
    allelic fraction of ≈0.31 (AD 65,31 / 61,28 / 66,28) rather than the ≈0.5 expected of a germline
    heterozygote. Three clustered, co-phased changes at a consistent sub-heterozygous fraction is the
    signature of a divergent or mismapped haplotype, not of three independent events. (An earlier
@@ -992,7 +1077,7 @@
    allelic fraction that do the work here.
 Even if the deletion were real, a single allele of an autosomal recessive disorder is carrier status.
 Sanger sequencing or long reads would be needed before any clinical report.
-GNRHR chr4:67753920 C&gt;T — c.416G&gt;A p.Arg139His, Exomiser ACMG LIKELY_PATHOGENIC. A clean
+GNRHR chr4:67753920 `C&gt;T` — `c.416G&gt;A` p.Arg139His, Exomiser ACMG LIKELY_PATHOGENIC. A clean
 heterozygote (AD 28,32, DP 60) and ClinVar Pathogenic (VariationID 16030, multiple submitters, no
 conflicts) for hypogonadotropic hypogonadism 7 with or without anosmia (OMIM 146110) — an
 autosomal recessive condition, so a single allele is carrier status. The allele reaches 3.3% in
@@ -1000,7 +1085,7 @@
 finding, and GNRHR does not appear on the ACMG SF v3.2 secondary findings gene list (statement:
 PMID 37347242; gene table as reproduced by NCBI ClinVar, checked directly). Carrier status is not a reportable secondary finding, and the condition is unrelated
 to this child's phenotype.
-We chose to document the reasoning rather than submit these as secondary rows. They would not have
+We chose to document the reasoning rather than submit these as `secondary` rows. They would not have
 harmed the automated score, but reporting them as findings would be a clinically meaningful false
 positive.</t>
         </is>
@@ -1014,12 +1099,12 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>- Exomiser genome-wide run: **53 seconds** wall clock (32-core CPU, 16 GB JVM heap).
+          <t>- Exomiser genome-wide run: 53 seconds wall clock (32-core CPU, 16 GB JVM heap).
 - Twelve robustness controls: about 11 minutes total.
 - Targeted panel with REST annotation: under 5 minutes, dominated by API latency.
 - Mosaicism analysis: about 10 minutes of `bcftools` streaming.
 - One-off setup: ≈55 GB of Exomiser reference data downloaded and extracted.
-- **Marginal compute cost is effectively zero** — a commodity workstation, no GPU, no cloud instance.
+- Marginal compute cost is effectively zero — a commodity workstation, no GPU, no cloud instance.
   Reproducing this on a laptop is realistic: only the 315 MB VCF and the phenotype document are
   needed, not the 85 GB of raw reads.</t>
         </is>
@@ -1035,41 +1120,38 @@
         <is>
           <t>We used two independent analyses and required them to converge.
 The primary analysis was hypothesis-free: Exomiser 15.1.0 (data 2602, hg38) on the complete proband
-VCF — 4,740,790 PASS variants — driven only by the eight HPO terms taken verbatim from the clinic. No gene panel, candidate list or disease name entered the configuration. **BUB1B is
-the top-ranked gene of 3,139, and its recessive row is first among the 2,100 recessive-model rows,
-mapped by Exomiser to mosaic variegated aneuploidy syndrome (ORPHA:1052)**, both variants
-contributing. Its *dominant* row scores higher (0.5871 vs 0.5538) but is attached to somatic
-colorectal cancer; **we report the recessive row and call the dominant one an artefact.** The
-recessive interpretation comes from the disease's inheritance model and the two-allele architecture,
-not from the ranking.
+VCF — 4,740,790 PASS variants — driven only by the eight HPO terms taken verbatim from the clinic. No
+gene panel, candidate list or disease name entered the configuration. BUB1B is the top-ranked gene
+of 3,139, and its recessive row is first among the 2,100 recessive-model rows, mapped by Exomiser to
+mosaic variegated aneuploidy syndrome (ORPHA:1052), both variants contributing. Its *dominant* row
+scores higher (0.5871 vs 0.5538) but is attached to somatic colorectal cancer; we report the
+recessive row and call the dominant one an artefact.
 The confirmatory analysis was orthogonal: an 11-gene MVA panel from Ensembl, annotated through VEP,
-filtered for HIGH/MODERATE impact below 1% gnomAD AF. Of 1,532 variants three survived; two were in BUB1B, the only
-gene with two rare damaging alleles.
-Both routes converge on **NM_001211.6:c.2210T&gt;G p.Leu737Ter** (nonsense; ClinVar 533901
-Pathogenic/Likely pathogenic; gnomAD 9.98×10⁻⁵) and **c.3006T&gt;G p.Asn1002Lys** (missense; gnomAD
+filtered for HIGH/MODERATE impact below 1% gnomAD AF. Of 1,532 variants three survived, two of them in
+BUB1B, the only gene with two rare damaging alleles.
+Both routes converge on NM_001211.6:c.2210T&gt;G p.Leu737Ter (nonsense; ClinVar 533901
+Pathogenic/Likely pathogenic; gnomAD 9.98×10⁻⁵) and c.3006T&gt;G p.Asn1002Lys (missense; gnomAD
 8.99×10⁻⁷; not in ClinVar) — the truncating-plus-missense pattern of viable MVA1.
-**Twelve robustness controls; the phenotype comes out weaker than we claimed.**
-Leave-one-HPO-out keeps BUB1B on top in all eight runs; five verified-unrelated HPO terms also return
-it there (0.4187 against 0.5871); and under those unrelated terms Exomiser still maps the
-recessive row to mosaic variegated aneuploidy, so the disease assignment comes from the OMIM
-prioritiser, not the phenotype. The finding is **variant-driven and
-phenotype-consistent**: the phenotype moves the score by 0.1684 and changes nothing else. We do not
-express that as a percentage — the combination is non-linear and a share is not defined.
-**We then measured what this pipeline does when the answer is absent**, in a benchmark pre-registered
-in git before any case ran. Seven healthy GIAB
-genomes queried with the same eight terms top out at **0.5619 against our 0.5871** — a margin of
-0.025 on a null biased in our favour; the pre-registered 30-genome tier is still running, so that
-prediction is open. Planting the same two public ClinVar alleles into three unrelated healthy genomes
-reproduces 0.5871 and 0.4187 to four decimals, none of them carrying its own retained BUB1B allele. And substituting an **unclassified** BUB1B nonsense for the whitelisted one
-leaves the variant term at 1.0000 and moves the combined score only 0.0128 without losing the top
-position (ACMG PATHOGENIC → LIKELY_PATHOGENIC): the truncating consequence, not the database record,
-saturates the variant term.
-**Limitations.** Phase is not observable here: no parental sample, no alignments (a VCF was
-distributed, so no read-backed phaser can be run), 10,911 bp between the variants with no GATK phase
-tag, and neither they nor the only heterozygous site between them is in the 1000 Genomes panel.
-Our pipeline is insensitive to phase regardless. p.Asn1002Lys is functionally unproven and its
-predictors disagree (REVEL 0.472, AlphaMissense 0.923). The genome-wide run took 53 seconds without
-a GPU.</t>
+Robustness controls; the phenotype comes out weaker than we claimed. Leave-one-HPO-out keeps
+BUB1B on top in all eight runs; five verified-unrelated HPO terms also return it there in the proband's
+genome (0.3965 against 0.5871). The finding is variant-driven and phenotype-consistent: the phenotype moves the score by
+0.1906 and changes nothing else. The unrelated-HPO control had to be rebuilt twice; the version quoted in our submitted
+entry (0.4187) was contaminated by a term annotated to MVA2.
+We then measured what this pipeline does when the answer is absent, in a benchmark pre-registered
+in git before any case ran. Seven healthy GIAB genomes queried with the same eight terms top out at
+0.5619 against our 0.5871 — a margin of 0.025 on a null biased in our favour. The pre-registered
+30-genome 1000 Genomes tier has since finished: maximum 0.5207 (CDH1, HG01885), 0 of 30 above
+0.5871. Planting the same two public ClinVar alleles into three unrelated healthy genomes reproduces
+0.5871 and 0.3965 to four decimals — stability across the backgrounds tested, not independence from
+the genome — while the *rank* under the unrelated phenotype holds in only one of the three, which
+falsifies a pre-registered prediction we said we expected to fail. Substituting an unclassified
+BUB1B nonsense for the whitelisted one moves the combined score only 0.0128 without losing the top
+position: the truncating consequence, not the database record, saturates the variant term.
+Limitations. Phase is not observable here: no parental sample, no alignments (the challenge
+distributed a VCF and raw reads, not a BAM, and we did not realign), 10,911 bp between the variants
+with no phase tag, and none of the relevant sites is in the 1000 Genomes panel. Our pipeline is
+insensitive to phase regardless. p.Asn1002Lys is functionally unproven and its predictors disagree
+(REVEL 0.472, AlphaMissense 0.923). The genome-wide run took 53 seconds without a GPU.</t>
         </is>
       </c>
     </row>
@@ -1140,11 +1222,11 @@
       <c r="B8" s="3" t="inlineStr">
         <is>
           <t>We went from variant to candidate in five steps, and the third and fifth are where most candidates die.
-Step 1 — establish the lesion. Compound heterozygosity in BUB1B: c.2210T&gt;G p.Leu737Ter, a
-nonsense allele that removes the C-terminal 313 residues, including the kinase domain (UniProt O60566 annotates it at 766–1050), paired with c.3006T&gt;G p.Asn1002Lys inside that domain. Loss of function, matching
+Step 1 — establish the lesion. Compound heterozygosity in BUB1B: `c.2210T&gt;G` p.Leu737Ter, a
+nonsense allele that removes the C-terminal 313 residues, including the kinase domain (UniProt O60566 annotates it at 766–1050), paired with `c.3006T&gt;G` p.Asn1002Lys inside that domain. Loss of function, matching
 the truncating-plus-missense pattern of viable MVA1: a null allele with a hypomorphic one. Reading the pair as null-plus-hypomorph is our reading of the human truncating-plus-missense pattern (PMID 20516114), which does not state that complete biallelic loss is lethal, and neither do we; the separate prediction that p.Asn1002Lys retains more residual function than L1012P comes from the Sieben mouse series (PMID 31738183), not from 20516114.
 Step 2 — follow the mechanism downstream, not at the lesion. No approved drug restores BubR1.
-We therefore asked what the lesion produces that is druggable. The chain is: weakened spindle
+We therefore asked what the lesion *produces* that is druggable. The chain is: weakened spindle
 assembly checkpoint → chromosome mis-segregation → constitutional aneuploidy → stoichiometric
 imbalance of protein complexes → proteotoxic stress. The last link is the one with approved drugs
 against it.
@@ -1155,7 +1237,7 @@
 | 1 | Regulatory | Approved for marketing? |
 | 2 | Mechanistic | Does it address the actual lesion or its consequence? |
 | 3 | Pharmacokinetic | Is Cmax ≥ the effective in vitro concentration? |
-| 4 | Patient-specific safety | Compatible with this child's comorbidities? |
+| 4 | Patient-specific safety | Compatible with *this* child's comorbidities? |
 | 5 | Direction of effect | Does it avoid increasing mis-segregation in survivors? |
 Step 4 — apply them, and report what dies. Metformin — the candidate the literature points to,
 descending from the AICAR hit of Tang et al. (PMID 21315436) — fails filter 3: therapeutic plasma
@@ -1165,10 +1247,10 @@
 inhibitors and reversine fail filter 5 by construction: they weaken a checkpoint that is already
 insufficient.
 Step 5 — the survivor, with its stopping condition. Bortezomib passes filters 1–3 and fails
-filter 4 for this child, which is a patient-specific verdict rather than a property of the drug.
+filter 4 *for this child*, which is a patient-specific verdict rather than a property of the drug.
 We state the condition under which it would become appropriate — an MVA patient with an active
 tumour, where the comparator is cytotoxic chemotherapy rather than nothing — and we propose an
-experiment — an eight-week assay window, about twelve weeks from a fresh biopsy — that could fail to support the dependency in this child's own cells. It would not, on its own, close the tumour-board question, and we say so where we describe it.</t>
+experiment — an eight-week assay window, 12–16 weeks from a fresh biopsy because establishing the fibroblast line takes 4–8 weeks on its own — that could fail to support the dependency in this child's own cells. It would not, on its own, close the tumour-board question, and we say so where we describe it.</t>
         </is>
       </c>
     </row>
@@ -1186,10 +1268,10 @@
 - OpenAI, Codex (gpt-5.6), Plus plan, "Improve the model for everyone" disabled.
 - xAI Grok 4.6 via Cursor, Pro plan, Privacy Mode enabled (zero data retention at Cursor
   and at the underlying model providers).
-- Piper TTS (en_US-ryan-high) — open-source, run locally with no cloud service and no API key.
+- Piper TTS (`en_US-ryan-high`) — open-source, run locally with no cloud service and no API key.
   Used only to narrate the pitch video; not a commercial service, listed for completeness.
 No block of the VCF and no genotype table was ever sent to a language model. Genomic work ran on
-local tools (bcftools, Exomiser) and on annotation APIs — Ensembl VEP and ClinVar — that the
+local tools (`bcftools`, Exomiser) and on annotation APIs — Ensembl VEP and ClinVar — that the
 hackathon policy names as acceptable.</t>
         </is>
       </c>
@@ -1228,8 +1310,8 @@
 2. Adversarial review by independent models. Two different language models were asked to attack
    our own drafts. They found, among others, a claim of ours that contradicted our own data file:
    the report stated that Tang et al. used only stable trisomies, when our extraction record shows
-   Figure 6 of that paper tests Bub1b^H/H hypomorphic MEFs. Corrected. All review rounds are in
-   evidencia/.
+   Figure 6 of that paper tests *Bub1b*^H/H hypomorphic MEFs. Corrected. All review rounds are in
+   `evidencia/`.
 3. Pharmacokinetic arithmetic, redone by hand. Each Cmax was converted from ng/mL to molar using
    the molecular weight, against the FDA label section cited. This surfaced that our own margin used
    the ceiling of a label interval (89–120 ng/mL) rather than the interval; corrected to 5.8–7.8×.</t>
@@ -1244,7 +1326,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Publicly available sources only. No proprietary drug/target databases or data sources were used.</t>
+          <t>Publicly available sources only. No proprietary data.</t>
         </is>
       </c>
     </row>
@@ -1308,10 +1390,20 @@
 no published functional assay, and its in-silico predictors disagree (REVEL 0.472, AlphaMissense
 0.923), which is why we let it stand as a VUS.
 We also asked whether aneuploidy burden could serve as a trial endpoint in these data, and computed
-that it cannot: simulating mean |BAF − 0.5| at DP 44 puts the detection limit at ~14% of cells for a
-clonal trisomy (16% under a stricter 2-SD criterion, against a measured between-chromosome SD of
-0.0035), while variegation leaves each chromosome at 1–2% — 7–16× below it. That constrains
-any proposal whose outcome depends on measuring aneuploidy from bulk sequencing.</t>
+that it cannot. A first-order calculation — mean |BAF − 0.5| at DP 44 against a measured
+between-chromosome SD of 0.0035 — puts the detection limit at ~14% of cells for a clonal trisomy (16%
+under a stricter 2-SD criterion). A later calibrated simulation (Ψ over 125-site windows, Monte Carlo
+null) improves that to 2.07% at an overdispersion κ = 2; that is a *simulated* limit conditional on
+κ, not a measured sensitivity, and it places variegation's 1–2% per chromosome at the edge of what is
+achievable rather than far below it. The argument that does not depend on any limit is
+non-identifiability: for a perfectly balanced variegated mixture, mean copy number is exactly 2 and
+mean allele fraction exactly 0.5 by symmetry, and simulated detection stays at the 0.1–0.2%
+false-positive rate even with 40% of cells aneuploid. That proof covers the balanced mixture we
+modelled, not every possible MVA genome, and it is enough to disqualify the endpoint.
+We ran the calibrated statistic on the proband and withdrew the result: the pre-registered
+threshold fires on all 22 autosomes, which indicates a null model that does not fit these data, and the
+pre-registered external control came back not conclusive because the control genomes were called
+differently from the proband. We report no clinical negative for this child.</t>
         </is>
       </c>
     </row>
@@ -1326,7 +1418,8 @@
           <t>Approximately 30 hours of analyst time over two days (28–29 August 2026), of which the large majority
 went to literature verification and adversarial review rather than to computation. Compute was
 negligible: the genome-wide prioritisation ran in 53 seconds on a commodity workstation with no GPU,
-and the eleven robustness controls in about ten minutes.</t>
+and the robustness controls in about ten minutes. Later rounds added the pre-registered DepMap,
+benchmark, phase, power and mosaicism-control analyses, all CPU-only and on public data.</t>
         </is>
       </c>
     </row>
@@ -1342,38 +1435,39 @@
 downstream — weakened spindle assembly checkpoint, mis-segregation, constitutional aneuploidy,
 stoichiometric protein imbalance, proteotoxic stress — and asked which approved agent acts on the
 last link.
-We then applied five filters instead of the usual two. Beyond "is it approved" and "is the
-mechanism plausible", we added a pharmacokinetic filter (does the achievable Cmax reach the
-concentration effective in vitro?), a patient-specific safety filter, and a direction-of-effect
-filter (does the drug increase mis-segregation among survivors?). Filters three and five are rarely
-applied and eliminate the most candidates.
-Metformin, the candidate the literature points to, dies on filter three. Therapeutic plasma
-levels are micromolar while complex I inhibition requires millimolar (PMID 37343530) — roughly a
-thousand-fold gap. We state what kind of number that is: for metformin no aneuploidy-selective EC50
-exists, so this is a comparison between concentration ranges, not the same quantity as a measured
-Cmax/EC50 ratio. We note what cuts the other way: AICAR's selectivity does reproduce in human cells
-(PMID 22890317), but that paper does not test metformin, and AICAR is not approved.
-Bortezomib survives filters one to three. Aneuploid cells mitigate proteotoxic stress by
-increasing protein degradation and are correspondingly sensitive to proteasome inhibition; aneuploidy
-level was significantly associated with multiple myeloma patients' response to proteasome inhibitors
-(Ippolito 2024, PMID 39247952), on cohorts small enough (8 complete responders vs 50 progressive)
-that we treat it as motivation, not prediction. The concentration reaches: EC50
-below 40 nM in highly aneuploid lines against a label Cmax of 89–120 ng/mL (231–312 nM) at
-1.3 mg/m² IV — a margin of 5.8–7.8× on total drug. The subcutaneous route does not pass once protein binding
-is considered, and we say so.
+We applied five filters instead of the usual two. Beyond "is it approved" and "is the mechanism
+plausible", we added a pharmacokinetic filter (does the achievable Cmax reach the concentration
+effective in vitro?), a patient-specific safety filter, and a direction-of-effect filter (does the drug
+increase mis-segregation among survivors?).
+Metformin, the candidate the literature points to, dies on filter three: therapeutic plasma levels are
+micromolar while complex I inhibition requires millimolar (PMID 37343530). AICAR's selectivity does
+reproduce in human cells (PMID 22890317), but that paper does not test metformin, and AICAR is not
+approved.
+Bortezomib survives filters one to three. Aneuploid cells depend on increased protein degradation, and
+aneuploidy level was associated with multiple myeloma patients' response to proteasome inhibitors
+(Ippolito 2024, PMID 39247952), on cohorts small enough (8 complete responders vs 50 progressive) that
+we treat it as motivation, not prediction. An EC50 below 40 nM in highly aneuploid lines against a
+label Cmax of 89–120 ng/mL (231–312 nM) at 1.3 mg/m² IV gives a margin of 5.8–7.8× on total plasma
+drug at a peak — not free or intratumoral drug, and 312 nM is the top of a label interval, not a
+validated clinical threshold.
 It then fails filter four for this child: motor neuropathy in 8% of paediatric patients, on top of
-existing skeletal muscle atrophy. But filter four is patient-specific.
-For an MVA patient with an active malignancy — where the comparator is cytotoxic chemotherapy rather
-than nothing — the balance inverts, and biallelic BUB1B carries a high risk of embryonal tumours. Our
-deliverable is that answer prepared in advance, with its margin and its stopping rule.
-Strengths. Every candidate is killed or kept by a stated criterion, including our own. We report an antagonism a combination-minded team could walk into: reducing translation protects
-CIN cells from proteasome inhibition (PMID 31530568), so mTOR inhibitors would be predicted to
-antagonise rather than synergise. The framework transfers to any rare disease.
+existing skeletal muscle atrophy. But filter four is patient-specific. For an MVA patient with an
+active malignancy — where the comparator is cytotoxic chemotherapy — the balance
+inverts, and biallelic BUB1B carries a high risk of embryonal tumours. Our deliverable is that answer
+prepared in advance, with its margin and its stopping rule.
+Strengths. Every candidate is killed or kept by a stated criterion, including our own; this is not an
+exhaustive screen, and §8 of the report lists what we excluded. We report an antagonism a
+combination-minded team could walk into: reducing translation protects CIN cells from proteasome
+inhibition (PMID 31530568), so mTOR inhibitors would be predicted to antagonise, not synergise. The
+framework transfers to any rare disease; applied to MVA2 and MVA3 it returns different verdicts.
 Limitations. The proteasome dependency is established in cancer aneuploidy, not constitutional
-mosaicism; whether it transfers is precisely what our eight-week experiment tests, and we
-have not assumed it. The EC50 is a conservative bound read from a figure panel. Phase is unproven and, we show, unobservable in these data; parental genotyping is the cheapest experiment here.
-And no disease-modifying drug can be recommended from these data today — what most changes his
-prognosis now is surveillance, not a molecule.</t>
+mosaicism; whether it transfers is what our proposed experiment tests. Our
+own pre-registered DepMap analysis found the association attenuated in solid lineages, the lineage of
+this child's tumour. The 0.897 power figure belongs to an idealised simulation with an *assumed*
+fourfold selectivity, not a validated estimate. The EC50 is a conservative bound read from a figure
+panel. Phase is unproven and unobservable in these data; parental genotyping is the cheapest
+informative experiment. No disease-modifying drug can be recommended from these data today — what most
+changes his prognosis now is surveillance, not a molecule.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
AI declaration: the narration is Qwen3-TTS now, not Piper
The methods form and both write-ups still named Piper TTS after the video was re-narrated with
Qwen3-TTS. Corrected in Q23 (Track 1), Q3 (Track 2), the internal note and the xlsx, with the
speech-recognition check on the generated clips stated alongside it.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Bin1pbSawAwvE2SkU7oJeK
</commit_message>
<xml_diff>
--- a/submission/methods_description_form_ciberpty.xlsx
+++ b/submission/methods_description_form_ciberpty.xlsx
@@ -927,9 +927,12 @@
 - OpenAI, Codex (gpt-5.6), Plus plan, "Improve the model for everyone" disabled.
 - xAI Grok 4.6 via Cursor, Pro plan, Privacy Mode enabled (zero data retention at Cursor
   and at the underlying model providers).
-- Piper TTS (`en_US-ryan-high`) — open-source, run entirely on local hardware with no cloud
+- Qwen3-TTS 1.7B VoiceDesign — open-weights, run entirely on local hardware (CPU) with no cloud
   service and no API key. Used only to narrate the pitch video. Listed for completeness; it is not a
-  commercial service.
+  commercial service. Every generated clip was transcribed by a local speech recogniser and diffed
+  against the written script before the video was assembled (`video/tts_verify.py`), because a
+  speech model of this kind can drop or alter a word silently — it did so once, and the affected
+  line was rewritten and re-generated.
 How these tools were used, and how they were not. The language models were used for literature
 retrieval and citation checking, for adversarial review of our own drafts, and for writing. They were
 also used against us on purpose: two independent models were asked to attack our reports, and the
@@ -1309,8 +1312,10 @@
 - OpenAI, Codex (gpt-5.6), Plus plan, "Improve the model for everyone" disabled.
 - xAI Grok 4.6 via Cursor, Pro plan, Privacy Mode enabled (zero data retention at Cursor
   and at the underlying model providers).
-- Piper TTS (`en_US-ryan-high`) — open-source, run locally with no cloud service and no API key.
-  Used only to narrate the pitch video; not a commercial service, listed for completeness.
+- Qwen3-TTS 1.7B VoiceDesign — open-weights, run locally on CPU with no cloud service and no API
+  key. Used only to narrate the pitch video; not a commercial service, listed for completeness. Each
+  clip was transcribed by a local recogniser and diffed against the written script before assembly,
+  because this class of model can alter a word silently.
 No block of the VCF and no genotype table was ever sent to a language model. Genomic work ran on
 local tools (`bcftools`, Exomiser) and on annotation APIs — Ensembl VEP and ClinVar — which return
 public annotation for submitted coordinates and acquire no rights over the input. The policy does not

</xml_diff>

<commit_message>
Transfer MVA-Replay to TRIP13 from a fresh clone; trametinib row; form and declaration sync
- replay/TRANSFER_TRIP13.md: results appended under the pre-registration (ee7a050).
  Scientific: rank 1 in 3/3 at 0.8332, unspiked absent/0, unrelated rank 1/2/3.
  Operational: tests did NOT run from a bare checkout (test fixed, tool untouched);
  README_TOOL requirements were three items short (now listed); name-prefix collision documented.
- Track 2 report: trametinib in the §3.3 table (PMID 39251587 abstract filed), §9 transfer bullet,
  paths to report/TRANSFER_MVA2_MVA3.md and the methods appendix.
- Track 1 Q11 no longer states a control count; Q3/Q23 name both Claude models used.
- PDFs rebuilt (23 + 53 pp.), xlsx cells B10/B18 and B9 synced, verifier: todo cuadra.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UCMRXDY3BR99D9KJ9SbKBz
</commit_message>
<xml_diff>
--- a/submission/methods_description_form_ciberpty.xlsx
+++ b/submission/methods_description_form_ciberpty.xlsx
@@ -922,7 +922,7 @@
       <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Commercially-available generative AI was used. Provider, plan and relevant setting for each:
-- Anthropic, Claude Opus via Claude Code, Max subscription plan, model-improvement data
+- Anthropic, Claude Opus and Claude Fable 5.1 via Claude Code, Max subscription plan, model-improvement data
   sharing disabled in account privacy settings.
 - OpenAI, Codex (gpt-5.6), Plus plan, "Improve the model for everyone" disabled.
 - xAI Grok 4.6 via Cursor, Pro plan, Privacy Mode enabled (zero data retention at Cursor
@@ -943,8 +943,7 @@
 return public annotation for submitted coordinates and acquire no rights over the input. The policy
 does not name these services; we read them as satisfying the two conditions it does set, namely no
 training on inputs or outputs and limited retention. What the models saw were named variants, HPO
-terms and reasoning: exactly the category the policy classifies as a "finding" and permits retaining.
----</t>
+terms and reasoning: exactly the category the policy classifies as a "finding" and permits retaining.</t>
         </is>
       </c>
     </row>
@@ -1139,7 +1138,8 @@
       <c r="B18" s="3" t="inlineStr">
         <is>
           <t>- Exomiser genome-wide run: 53 seconds wall clock (32-core CPU, 16 GB JVM heap).
-- Twelve robustness controls: about 11 minutes total.
+- Robustness controls (the families listed under Robustness controls above, one Exomiser run each): about
+  a minute per run, roughly 11 minutes in total.
 - Targeted panel with REST annotation: under 5 minutes, dominated by API latency.
 - Mosaicism first-order BAF scan: about 10 minutes of `bcftools` streaming.
 - Mosaicism null calibration (40,000 Monte Carlo replicates per cell, eight window sizes): run with
@@ -1307,7 +1307,7 @@
       <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Commercially-available generative AI was used. Provider, plan and relevant setting for each:
-- Anthropic, Claude Opus via Claude Code, Max subscription plan, model-improvement data
+- Anthropic, Claude Opus and Claude Fable 5.1 via Claude Code, Max subscription plan, model-improvement data
   sharing disabled in account privacy settings.
 - OpenAI, Codex (gpt-5.6), Plus plan, "Improve the model for everyone" disabled.
 - xAI Grok 4.6 via Cursor, Pro plan, Privacy Mode enabled (zero data retention at Cursor

</xml_diff>

<commit_message>
Four-parameter power follow-up, pre-registered and run: power 0.167 at n = 3, not 0.897; 12 cultures per arm at f = 0.30
Parallel run over 32 cores (Amendment 1, committed before any number was seen; 397 s). Fitting never
failed; the biological variability is the cost, so two of four predictions were falsified and are
reported. The n = 3 and n = 14 branches are retired from §6 of both parts; 0.897 stays as the optimistic
two-parameter reference; the Track 2 abstract states the new figure (496 words). Micronucleus criterion
is now a decision rule with a confidence interval. Verifier anchors the new numbers to resultados_4p.json
(31 facts, all match). Handoff updated: changes #3 and #5 complete.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UCMRXDY3BR99D9KJ9SbKBz
</commit_message>
<xml_diff>
--- a/submission/methods_description_form_ciberpty.xlsx
+++ b/submission/methods_description_form_ciberpty.xlsx
@@ -1519,8 +1519,8 @@
 Limitations. The proteasome dependency is established in cancer aneuploidy, not constitutional
 mosaicism; whether it transfers is what our proposed experiment tests. Our
 own pre-registered DepMap analysis found the association attenuated in solid lineages, the lineage of
-this child's tumour. The 0.897 power figure belongs to an idealised simulation with an assumed
-fourfold selectivity, not a validated estimate. The EC50 is a conservative bound read from a figure
+this child's tumour. Under the pre-registered four-parameter model with biological variability the assay
+has power 0.17 at n = 3 and needs about 12 cultures per arm. The EC50 is a conservative bound read from a figure
 panel. Phase is unproven and unobservable in these data; parental genotyping is the cheapest
 informative experiment. No disease-modifying drug can be recommended from these data today — what most
 changes his prognosis now is surveillance, not a molecule.</t>

</xml_diff>